<commit_message>
Add Apollo decision-maker roster (95 contacts) + update Batch 1 Excel
</commit_message>
<xml_diff>
--- a/market-research/I-MAK_Denmark_Batch1_Food.xlsx
+++ b/market-research/I-MAK_Denmark_Batch1_Food.xlsx
@@ -23,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -56,6 +56,11 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="13"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <i val="1"/>
+      <color rgb="002E5496"/>
     </font>
     <font>
       <i val="1"/>
@@ -126,7 +131,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -154,6 +159,7 @@
     <xf numFmtId="0" fontId="6" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -8675,15 +8681,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:G102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8694,51 +8701,69 @@
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>Role (target)</t>
+          <t>Role Category</t>
         </is>
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>First Name</t>
         </is>
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
-          <t>LinkedIn / Email</t>
+          <t>Last Name (masked)</t>
         </is>
       </c>
       <c r="E1" s="4" t="inlineStr">
         <is>
-          <t>Source</t>
+          <t>Exact Title</t>
         </is>
       </c>
       <c r="F1" s="4" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Full Name / Email / LinkedIn</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Carsoe (Carsoe Group A/S)</t>
+          <t>Gram Equipment A/S</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>CEO / Managing Director</t>
-        </is>
-      </c>
-      <c r="C2" s="5" t="inlineStr"/>
-      <c r="D2" s="5" t="inlineStr"/>
+          <t>CEO/MD</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Dirk</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Ha***g</t>
+        </is>
+      </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>TO ENRICH via Apollo.io</t>
+          <t>CEO Gram-Equipment A/S</t>
         </is>
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
         </is>
       </c>
     </row>
@@ -8750,115 +8775,180 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>CEO / Managing Director</t>
-        </is>
-      </c>
-      <c r="C3" s="7" t="inlineStr"/>
-      <c r="D3" s="7" t="inlineStr"/>
+          <t>Purchasing/Procurement</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>Peter</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>Ra***n</t>
+        </is>
+      </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>TO ENRICH via Apollo.io</t>
+          <t>Strategic Procurement Manager &amp; Lead</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>Frontmatec Group (SFK, Attec, Carometec, ITEC)</t>
+          <t>Gram Equipment A/S</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>CEO / Managing Director</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="5" t="inlineStr"/>
+          <t>R&amp;D</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Michael</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Co***s</t>
+        </is>
+      </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>TO ENRICH via Apollo.io</t>
+          <t>R&amp;D Manager</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>Attec Danmark A/S</t>
+          <t>Gram Equipment A/S</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>CEO / Managing Director</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr"/>
-      <c r="D5" s="7" t="inlineStr"/>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Jens</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>Ha***n</t>
+        </is>
+      </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>TO ENRICH via Apollo.io</t>
+          <t>Production Manager</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Aasted ApS</t>
+          <t>Cabinplant A/S</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>CEO / Managing Director</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr"/>
+          <t>CEO/MD (Owner)</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Jan</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Ha***n</t>
+        </is>
+      </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>TO ENRICH via Apollo.io</t>
+          <t>CFO, Co-owner</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>Sealing System 2024 A/S</t>
+          <t>Cabinplant A/S</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>CEO / Managing Director</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="inlineStr"/>
-      <c r="D7" s="7" t="inlineStr"/>
+          <t>Purchasing/Procurement</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Juergen</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Ju***n</t>
+        </is>
+      </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>TO ENRICH via Apollo.io</t>
+          <t>Procurement Manager</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
         </is>
       </c>
     </row>
@@ -8870,225 +8960,3353 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>CEO / Managing Director</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr"/>
-      <c r="D8" s="5" t="inlineStr"/>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Michael</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Pe***n</t>
+        </is>
+      </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>TO ENRICH via Apollo.io</t>
+          <t>Engineering Manager - Processing</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>Uni-Food Technic A/S</t>
+          <t>Cabinplant A/S</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>CEO / Managing Director</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="inlineStr"/>
-      <c r="D9" s="7" t="inlineStr"/>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Henrik</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>So***d</t>
+        </is>
+      </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>TO ENRICH via Apollo.io</t>
+          <t>Production Manager</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Kroma A/S</t>
+          <t>Carsoe (Carsoe Group A/S)</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>CEO / Managing Director</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr"/>
-      <c r="D10" s="5" t="inlineStr"/>
+          <t>CEO/MD</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Soren</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Kl***o</t>
+        </is>
+      </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>TO ENRICH via Apollo.io</t>
+          <t>CEO</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>Primodan A/S</t>
+          <t>Carsoe (Carsoe Group A/S)</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>CEO / Managing Director</t>
-        </is>
-      </c>
-      <c r="C11" s="7" t="inlineStr"/>
-      <c r="D11" s="7" t="inlineStr"/>
+          <t>Technical Director</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Henrik</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>Po***n</t>
+        </is>
+      </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>TO ENRICH via Apollo.io</t>
+          <t>CTO</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>SiccaDania A/S</t>
+          <t>Carsoe (Carsoe Group A/S)</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>CEO / Managing Director</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr"/>
-      <c r="D12" s="5" t="inlineStr"/>
+          <t>Purchasing/Procurement</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Doris</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Ha***n</t>
+        </is>
+      </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>TO ENRICH via Apollo.io</t>
+          <t>Procurement &amp; Logistics Manager</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>Landia A/S</t>
+          <t>Carsoe (Carsoe Group A/S)</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>CEO / Managing Director</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="inlineStr"/>
-      <c r="D13" s="7" t="inlineStr"/>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Magnus</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>He***d</t>
+        </is>
+      </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>TO ENRICH via Apollo.io</t>
+          <t>Manager of Mechanical Engineering</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Scansteel foodtech A/S</t>
+          <t>KM Fish Machinery A/S</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>CEO / Managing Director</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr"/>
-      <c r="D14" s="5" t="inlineStr"/>
+          <t>CEO/MD</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Soren</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Kl***o</t>
+        </is>
+      </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>TO ENRICH via Apollo.io</t>
+          <t>CEO (shared Carsoe org)</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>JS Proputec A/S</t>
+          <t>KM Fish Machinery A/S</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>CEO / Managing Director</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="inlineStr"/>
-      <c r="D15" s="7" t="inlineStr"/>
+          <t>Purchasing/Procurement</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Doris</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>Ha***n</t>
+        </is>
+      </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>TO ENRICH via Apollo.io</t>
+          <t>Procurement &amp; Logistics Manager (shared Carsoe org)</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G15" s="7" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
+          <t>Uni-Food Technic A/S</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>CEO/MD (Owner)</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Jeppe</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Ch***n</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Chief Executive Officer, Owner</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>Uni-Food Technic A/S</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Michael</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>Ha***n</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>Production Manager</t>
+        </is>
+      </c>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Kaj Olesen A/S</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>CEO/MD</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Jacob</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>Ol***n</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>IRAS A/S</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>CEO/MD (Owner)</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>Peter</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>Ra***n</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>DSI Freezing Solutions / DSI Dantech A/S</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Supply Chain</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Hans</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Vi***d</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>Supply Chain Director (interim)</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>DSI Freezing Solutions / DSI Dantech A/S</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>Anders</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>Ch***n</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>Production Manager</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Qupaq A/S</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>CEO/MD</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Christian</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Bo***s</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>Chief Executive Officer</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>Globaq Solutions (ex-Billund Aquaculture)</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>Carlos</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>Ar***i</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>Engineering Manager</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Primodan A/S</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>CEO/MD</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Lars</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>He***n</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>Primodan A/S</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>Tommy</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>Ol***n</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>Production Manager</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>SiccaDania A/S</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>CEO/MD</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Lone</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Ho***t</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>CEO SiccaDania Holding</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>SiccaDania A/S</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
+        <is>
+          <t>Willy</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>Ma***k</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>Engineering Manager</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Tetra Pak Hoyer A/S</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Lasse</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>Je***n</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>Production Manager</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>Tetra Pak Hoyer A/S</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="C29" s="7" t="inlineStr">
+        <is>
+          <t>Morten</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>Os***i</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>Engineering Manager</t>
+        </is>
+      </c>
+      <c r="F29" s="7" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G29" s="7" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Tetra Pak Hoyer A/S</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Purchasing/Procurement</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Allen</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Le***y</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>Senior Innovation Procurement Manager</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>Tetra Pak Hoyer A/S</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>R&amp;D</t>
+        </is>
+      </c>
+      <c r="C31" s="7" t="inlineStr">
+        <is>
+          <t>Soren</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>An***n</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="inlineStr">
+        <is>
+          <t>R&amp;D Project Manager</t>
+        </is>
+      </c>
+      <c r="F31" s="7" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G31" s="7" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>Tetra Pak Hoyer A/S</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>Supply Chain</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>Bente</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>Da***d</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>Supply Manager</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>Tetra Pak Hoyer A/S</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>Technical Director</t>
+        </is>
+      </c>
+      <c r="C33" s="7" t="inlineStr">
+        <is>
+          <t>(Mr.)</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>Ra***n</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>Technical Sales Director</t>
+        </is>
+      </c>
+      <c r="F33" s="7" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G33" s="7" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>GEA Process Engineering A/S (ex-Niro)</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>CEO/MD</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>Claus</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Th***n</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>Country Mgr Dir DACH &amp; Nordics NPE / MD GEA Liquid Technologies A/S</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>GEA Process Engineering A/S (ex-Niro)</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>Technical Director</t>
+        </is>
+      </c>
+      <c r="C35" s="7" t="inlineStr">
+        <is>
+          <t>Poul-Erik</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>Aa***d</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>Technical Director</t>
+        </is>
+      </c>
+      <c r="F35" s="7" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G35" s="7" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>GEA Process Engineering A/S (ex-Niro)</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>R&amp;D</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>Anders</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Re***n</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>Head of Digitalization and Automation R&amp;D</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>GEA Process Engineering A/S (ex-Niro)</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>Supply Chain</t>
+        </is>
+      </c>
+      <c r="C37" s="7" t="inlineStr">
+        <is>
+          <t>Lars</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>Ho***n</t>
+        </is>
+      </c>
+      <c r="E37" s="7" t="inlineStr">
+        <is>
+          <t>Senior Director Procurement &amp; Supply Chain</t>
+        </is>
+      </c>
+      <c r="F37" s="7" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G37" s="7" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>GEA Process Engineering A/S (ex-Niro)</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>Purchasing/Procurement</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>Rene</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Cl***n</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>Head of Procurement (interim), GEA Liquid Technology A/S</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G38" s="5" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>GEA Process Engineering A/S (ex-Niro)</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>Peter</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>Pl***t</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>Head of Project Engineering - Membrane Filtration</t>
+        </is>
+      </c>
+      <c r="F39" s="7" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G39" s="7" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SPX FLOW Danmark (APV)</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>Lis</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>Ra***n</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>Engineering Manager, Process Technology Membrane &amp; UHT</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G40" s="5" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>NDT - Nordic Dairy Technology ApS</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>CEO/MD</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>Stig</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="inlineStr">
+        <is>
+          <t>Pe***n</t>
+        </is>
+      </c>
+      <c r="E41" s="7" t="inlineStr">
+        <is>
+          <t>Chief Executive Officer</t>
+        </is>
+      </c>
+      <c r="F41" s="7" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G41" s="7" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Egatec A/S</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>CEO/MD</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>Rene</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Mo***r</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>Adm. Direktor / CEO</t>
+        </is>
+      </c>
+      <c r="F42" s="5" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G42" s="5" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="7" t="inlineStr">
+        <is>
+          <t>Egatec A/S</t>
+        </is>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>Tommy</t>
+        </is>
+      </c>
+      <c r="D43" s="7" t="inlineStr">
+        <is>
+          <t>Pe***n</t>
+        </is>
+      </c>
+      <c r="E43" s="7" t="inlineStr">
+        <is>
+          <t>Head of Engineering, Automation</t>
+        </is>
+      </c>
+      <c r="F43" s="7" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G43" s="7" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Frontmatec Group</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>Supply Chain</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>Thorbjorn</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>Be***n</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>Senior Director Supply Chain Europe</t>
+        </is>
+      </c>
+      <c r="F44" s="5" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G44" s="5" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="7" t="inlineStr">
+        <is>
+          <t>Frontmatec Group</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>R&amp;D</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>Thomas</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="inlineStr">
+        <is>
+          <t>La***n</t>
+        </is>
+      </c>
+      <c r="E45" s="7" t="inlineStr">
+        <is>
+          <t>R&amp;D Manager, Instruments</t>
+        </is>
+      </c>
+      <c r="F45" s="7" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G45" s="7" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>Scansteel foodtech A/S</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>CEO/MD</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>Henrik</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>Sa***g</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>CEO/Owner</t>
+        </is>
+      </c>
+      <c r="F46" s="5" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G46" s="5" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="7" t="inlineStr">
+        <is>
+          <t>Scansteel foodtech A/S</t>
+        </is>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>R&amp;D</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="inlineStr">
+        <is>
+          <t>Henrik</t>
+        </is>
+      </c>
+      <c r="D47" s="7" t="inlineStr">
+        <is>
+          <t>La***n</t>
+        </is>
+      </c>
+      <c r="E47" s="7" t="inlineStr">
+        <is>
+          <t>Project and R&amp;D Manager</t>
+        </is>
+      </c>
+      <c r="F47" s="7" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G47" s="7" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Scansteel foodtech A/S</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>Mohammad</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>Sa***y</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>Technical Engineering Manager</t>
+        </is>
+      </c>
+      <c r="F48" s="5" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G48" s="5" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="7" t="inlineStr">
+        <is>
+          <t>Fomaco A/S</t>
+        </is>
+      </c>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>CEO/MD</t>
+        </is>
+      </c>
+      <c r="C49" s="7" t="inlineStr">
+        <is>
+          <t>Sebastian</t>
+        </is>
+      </c>
+      <c r="D49" s="7" t="inlineStr">
+        <is>
+          <t>Mu***r</t>
+        </is>
+      </c>
+      <c r="E49" s="7" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="F49" s="7" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G49" s="7" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Fomaco A/S</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>Technical Director</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>Carsten</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>Gi***l</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>CTO</t>
+        </is>
+      </c>
+      <c r="F50" s="5" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G50" s="5" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="7" t="inlineStr">
+        <is>
+          <t>Fomaco A/S</t>
+        </is>
+      </c>
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="C51" s="7" t="inlineStr">
+        <is>
+          <t>Ole</t>
+        </is>
+      </c>
+      <c r="D51" s="7" t="inlineStr">
+        <is>
+          <t>Ni***n</t>
+        </is>
+      </c>
+      <c r="E51" s="7" t="inlineStr">
+        <is>
+          <t>Production Manager</t>
+        </is>
+      </c>
+      <c r="F51" s="7" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G51" s="7" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>JS Proputec A/S</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>CEO/MD</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>Morten</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>Br***g</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>Chief Executive Officer</t>
+        </is>
+      </c>
+      <c r="F52" s="5" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G52" s="5" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="7" t="inlineStr">
+        <is>
+          <t>JS Proputec A/S</t>
+        </is>
+      </c>
+      <c r="B53" s="7" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="C53" s="7" t="inlineStr">
+        <is>
+          <t>Bjarne</t>
+        </is>
+      </c>
+      <c r="D53" s="7" t="inlineStr">
+        <is>
+          <t>Je***n</t>
+        </is>
+      </c>
+      <c r="E53" s="7" t="inlineStr">
+        <is>
+          <t>Production Manager</t>
+        </is>
+      </c>
+      <c r="F53" s="7" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G53" s="7" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
           <t>BAADER Food Systems Denmark A/S (ex-LINCO)</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>CEO / Managing Director</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr"/>
-      <c r="D16" s="5" t="inlineStr"/>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>TO ENRICH via Apollo.io</t>
-        </is>
-      </c>
-      <c r="F16" s="5" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="12" t="inlineStr">
-        <is>
-          <t>NOTE: This tab is a template. Names + personal LinkedIn/email are not reliably public and are</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="12" t="inlineStr">
-        <is>
-          <t>reserved for an Apollo.io enrichment pass across all 49 companies (targets: CEO / Managing Director, Purchasing / Procurement Director, Engineering Manager, R&amp;D Manager, Production Manager, Technical Director, Supply Chain Director).</t>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>CEO/MD</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>Henning</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>Pe***n</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>Managing Director / CEO</t>
+        </is>
+      </c>
+      <c r="F54" s="5" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G54" s="5" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="7" t="inlineStr">
+        <is>
+          <t>BAADER Food Systems Denmark A/S (ex-LINCO)</t>
+        </is>
+      </c>
+      <c r="B55" s="7" t="inlineStr">
+        <is>
+          <t>R&amp;D</t>
+        </is>
+      </c>
+      <c r="C55" s="7" t="inlineStr">
+        <is>
+          <t>Michael</t>
+        </is>
+      </c>
+      <c r="D55" s="7" t="inlineStr">
+        <is>
+          <t>Ha***n</t>
+        </is>
+      </c>
+      <c r="E55" s="7" t="inlineStr">
+        <is>
+          <t>Head of R&amp;D</t>
+        </is>
+      </c>
+      <c r="F55" s="7" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G55" s="7" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>BAADER Food Systems Denmark A/S (ex-LINCO)</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>Danny</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>Od***e</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>Engineering Manager</t>
+        </is>
+      </c>
+      <c r="F56" s="5" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G56" s="5" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="7" t="inlineStr">
+        <is>
+          <t>BAADER Food Systems Denmark A/S (ex-LINCO)</t>
+        </is>
+      </c>
+      <c r="B57" s="7" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="C57" s="7" t="inlineStr">
+        <is>
+          <t>Niels</t>
+        </is>
+      </c>
+      <c r="D57" s="7" t="inlineStr">
+        <is>
+          <t>Th***n</t>
+        </is>
+      </c>
+      <c r="E57" s="7" t="inlineStr">
+        <is>
+          <t>Production Manager</t>
+        </is>
+      </c>
+      <c r="F57" s="7" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G57" s="7" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>BAADER Food Systems Denmark A/S (ex-LINCO)</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>Technical Director</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>Michael</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>Ba***g</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>Technical Director</t>
+        </is>
+      </c>
+      <c r="F58" s="5" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G58" s="5" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="7" t="inlineStr">
+        <is>
+          <t>Jorgensen Engineering A/S</t>
+        </is>
+      </c>
+      <c r="B59" s="7" t="inlineStr">
+        <is>
+          <t>CEO/MD</t>
+        </is>
+      </c>
+      <c r="C59" s="7" t="inlineStr">
+        <is>
+          <t>Mike</t>
+        </is>
+      </c>
+      <c r="D59" s="7" t="inlineStr">
+        <is>
+          <t>Go***a</t>
+        </is>
+      </c>
+      <c r="E59" s="7" t="inlineStr">
+        <is>
+          <t>Chief Executive Officer</t>
+        </is>
+      </c>
+      <c r="F59" s="7" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G59" s="7" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr">
+        <is>
+          <t>Jorgensen Engineering A/S</t>
+        </is>
+      </c>
+      <c r="B60" s="5" t="inlineStr">
+        <is>
+          <t>Technical Director</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>Thomas</t>
+        </is>
+      </c>
+      <c r="D60" s="5" t="inlineStr">
+        <is>
+          <t>La***n</t>
+        </is>
+      </c>
+      <c r="E60" s="5" t="inlineStr">
+        <is>
+          <t>Chief Technology Officer</t>
+        </is>
+      </c>
+      <c r="F60" s="5" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G60" s="5" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="7" t="inlineStr">
+        <is>
+          <t>Jorgensen Engineering A/S</t>
+        </is>
+      </c>
+      <c r="B61" s="7" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="C61" s="7" t="inlineStr">
+        <is>
+          <t>Jeppe</t>
+        </is>
+      </c>
+      <c r="D61" s="7" t="inlineStr">
+        <is>
+          <t>Jo***n</t>
+        </is>
+      </c>
+      <c r="E61" s="7" t="inlineStr">
+        <is>
+          <t>Engineering Manager</t>
+        </is>
+      </c>
+      <c r="F61" s="7" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G61" s="7" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr">
+        <is>
+          <t>Jorgensen Engineering A/S</t>
+        </is>
+      </c>
+      <c r="B62" s="5" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="inlineStr">
+        <is>
+          <t>Johnni</t>
+        </is>
+      </c>
+      <c r="D62" s="5" t="inlineStr">
+        <is>
+          <t>Ha***n</t>
+        </is>
+      </c>
+      <c r="E62" s="5" t="inlineStr">
+        <is>
+          <t>Production Manager</t>
+        </is>
+      </c>
+      <c r="F62" s="5" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G62" s="5" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="7" t="inlineStr">
+        <is>
+          <t>Haarslev Industries A/S</t>
+        </is>
+      </c>
+      <c r="B63" s="7" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="C63" s="7" t="inlineStr">
+        <is>
+          <t>Kaare</t>
+        </is>
+      </c>
+      <c r="D63" s="7" t="inlineStr">
+        <is>
+          <t>Ve***g</t>
+        </is>
+      </c>
+      <c r="E63" s="7" t="inlineStr">
+        <is>
+          <t>Engineering Centre Manager</t>
+        </is>
+      </c>
+      <c r="F63" s="7" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G63" s="7" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="inlineStr">
+        <is>
+          <t>Haarslev Industries A/S</t>
+        </is>
+      </c>
+      <c r="B64" s="5" t="inlineStr">
+        <is>
+          <t>Engineering (Automation)</t>
+        </is>
+      </c>
+      <c r="C64" s="5" t="inlineStr">
+        <is>
+          <t>Henrik</t>
+        </is>
+      </c>
+      <c r="D64" s="5" t="inlineStr">
+        <is>
+          <t>Je***n</t>
+        </is>
+      </c>
+      <c r="E64" s="5" t="inlineStr">
+        <is>
+          <t>Engineering Centre Manager - Automation &amp; Control</t>
+        </is>
+      </c>
+      <c r="F64" s="5" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G64" s="5" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="7" t="inlineStr">
+        <is>
+          <t>Haarslev Industries A/S</t>
+        </is>
+      </c>
+      <c r="B65" s="7" t="inlineStr">
+        <is>
+          <t>Sales Engineering</t>
+        </is>
+      </c>
+      <c r="C65" s="7" t="inlineStr">
+        <is>
+          <t>Hamed</t>
+        </is>
+      </c>
+      <c r="D65" s="7" t="inlineStr">
+        <is>
+          <t>Sh***i</t>
+        </is>
+      </c>
+      <c r="E65" s="7" t="inlineStr">
+        <is>
+          <t>Sales Engineering Manager</t>
+        </is>
+      </c>
+      <c r="F65" s="7" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G65" s="7" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="inlineStr">
+        <is>
+          <t>Daniatech ApS / SD Mixing (SiccaDania)</t>
+        </is>
+      </c>
+      <c r="B66" s="5" t="inlineStr">
+        <is>
+          <t>CEO/MD</t>
+        </is>
+      </c>
+      <c r="C66" s="5" t="inlineStr">
+        <is>
+          <t>Jens</t>
+        </is>
+      </c>
+      <c r="D66" s="5" t="inlineStr">
+        <is>
+          <t>An***n</t>
+        </is>
+      </c>
+      <c r="E66" s="5" t="inlineStr">
+        <is>
+          <t>Managing Director</t>
+        </is>
+      </c>
+      <c r="F66" s="5" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G66" s="5" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="7" t="inlineStr">
+        <is>
+          <t>Daniatech ApS / SD Mixing (SiccaDania)</t>
+        </is>
+      </c>
+      <c r="B67" s="7" t="inlineStr">
+        <is>
+          <t>R&amp;D/Technical</t>
+        </is>
+      </c>
+      <c r="C67" s="7" t="inlineStr">
+        <is>
+          <t>Gorm</t>
+        </is>
+      </c>
+      <c r="D67" s="7" t="inlineStr">
+        <is>
+          <t>Kj***f</t>
+        </is>
+      </c>
+      <c r="E67" s="7" t="inlineStr">
+        <is>
+          <t>Technology Owner, UHT &amp; Thermal Processing</t>
+        </is>
+      </c>
+      <c r="F67" s="7" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G67" s="7" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="5" t="inlineStr">
+        <is>
+          <t>SANOVO Technology A/S</t>
+        </is>
+      </c>
+      <c r="B68" s="5" t="inlineStr">
+        <is>
+          <t>CEO/MD</t>
+        </is>
+      </c>
+      <c r="C68" s="5" t="inlineStr">
+        <is>
+          <t>Michael</t>
+        </is>
+      </c>
+      <c r="D68" s="5" t="inlineStr">
+        <is>
+          <t>Mi***v</t>
+        </is>
+      </c>
+      <c r="E68" s="5" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="F68" s="5" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G68" s="5" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="7" t="inlineStr">
+        <is>
+          <t>SANOVO Technology A/S</t>
+        </is>
+      </c>
+      <c r="B69" s="7" t="inlineStr">
+        <is>
+          <t>R&amp;D</t>
+        </is>
+      </c>
+      <c r="C69" s="7" t="inlineStr">
+        <is>
+          <t>Martin</t>
+        </is>
+      </c>
+      <c r="D69" s="7" t="inlineStr">
+        <is>
+          <t>So***n</t>
+        </is>
+      </c>
+      <c r="E69" s="7" t="inlineStr">
+        <is>
+          <t>R&amp;D Manager</t>
+        </is>
+      </c>
+      <c r="F69" s="7" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G69" s="7" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="5" t="inlineStr">
+        <is>
+          <t>SANOVO Technology A/S</t>
+        </is>
+      </c>
+      <c r="B70" s="5" t="inlineStr">
+        <is>
+          <t>Engineering (Electrical)</t>
+        </is>
+      </c>
+      <c r="C70" s="5" t="inlineStr">
+        <is>
+          <t>Henrik</t>
+        </is>
+      </c>
+      <c r="D70" s="5" t="inlineStr">
+        <is>
+          <t>Mo***r</t>
+        </is>
+      </c>
+      <c r="E70" s="5" t="inlineStr">
+        <is>
+          <t>Product Owner, Electrical</t>
+        </is>
+      </c>
+      <c r="F70" s="5" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G70" s="5" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="7" t="inlineStr">
+        <is>
+          <t>Scanvaegt Systems A/S</t>
+        </is>
+      </c>
+      <c r="B71" s="7" t="inlineStr">
+        <is>
+          <t>CEO/MD</t>
+        </is>
+      </c>
+      <c r="C71" s="7" t="inlineStr">
+        <is>
+          <t>Jan</t>
+        </is>
+      </c>
+      <c r="D71" s="7" t="inlineStr">
+        <is>
+          <t>El***d</t>
+        </is>
+      </c>
+      <c r="E71" s="7" t="inlineStr">
+        <is>
+          <t>Adm. Direktor / CEO</t>
+        </is>
+      </c>
+      <c r="F71" s="7" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G71" s="7" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="5" t="inlineStr">
+        <is>
+          <t>Scanvaegt Systems A/S</t>
+        </is>
+      </c>
+      <c r="B72" s="5" t="inlineStr">
+        <is>
+          <t>R&amp;D</t>
+        </is>
+      </c>
+      <c r="C72" s="5" t="inlineStr">
+        <is>
+          <t>Simon</t>
+        </is>
+      </c>
+      <c r="D72" s="5" t="inlineStr">
+        <is>
+          <t>So***d</t>
+        </is>
+      </c>
+      <c r="E72" s="5" t="inlineStr">
+        <is>
+          <t>R&amp;D Team Manager</t>
+        </is>
+      </c>
+      <c r="F72" s="5" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G72" s="5" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="7" t="inlineStr">
+        <is>
+          <t>Scanvaegt Systems A/S</t>
+        </is>
+      </c>
+      <c r="B73" s="7" t="inlineStr">
+        <is>
+          <t>R&amp;D (Project)</t>
+        </is>
+      </c>
+      <c r="C73" s="7" t="inlineStr">
+        <is>
+          <t>Niels</t>
+        </is>
+      </c>
+      <c r="D73" s="7" t="inlineStr">
+        <is>
+          <t>Hu***e</t>
+        </is>
+      </c>
+      <c r="E73" s="7" t="inlineStr">
+        <is>
+          <t>Project Manager R&amp;D</t>
+        </is>
+      </c>
+      <c r="F73" s="7" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G73" s="7" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="5" t="inlineStr">
+        <is>
+          <t>Schur Technology A/S (Schur Group)</t>
+        </is>
+      </c>
+      <c r="B74" s="5" t="inlineStr">
+        <is>
+          <t>CEO/MD</t>
+        </is>
+      </c>
+      <c r="C74" s="5" t="inlineStr">
+        <is>
+          <t>Hans</t>
+        </is>
+      </c>
+      <c r="D74" s="5" t="inlineStr">
+        <is>
+          <t>Sc***r</t>
+        </is>
+      </c>
+      <c r="E74" s="5" t="inlineStr">
+        <is>
+          <t>Chief Executive Officer</t>
+        </is>
+      </c>
+      <c r="F74" s="5" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G74" s="5" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="7" t="inlineStr">
+        <is>
+          <t>Schur Technology A/S (Schur Group)</t>
+        </is>
+      </c>
+      <c r="B75" s="7" t="inlineStr">
+        <is>
+          <t>Purchasing/Procurement</t>
+        </is>
+      </c>
+      <c r="C75" s="7" t="inlineStr">
+        <is>
+          <t>Kasper</t>
+        </is>
+      </c>
+      <c r="D75" s="7" t="inlineStr">
+        <is>
+          <t>An***n</t>
+        </is>
+      </c>
+      <c r="E75" s="7" t="inlineStr">
+        <is>
+          <t>Procurement Manager</t>
+        </is>
+      </c>
+      <c r="F75" s="7" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G75" s="7" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="5" t="inlineStr">
+        <is>
+          <t>Schur Technology A/S (Schur Group)</t>
+        </is>
+      </c>
+      <c r="B76" s="5" t="inlineStr">
+        <is>
+          <t>Supply Chain</t>
+        </is>
+      </c>
+      <c r="C76" s="5" t="inlineStr">
+        <is>
+          <t>Ditte</t>
+        </is>
+      </c>
+      <c r="D76" s="5" t="inlineStr">
+        <is>
+          <t>Ch***n</t>
+        </is>
+      </c>
+      <c r="E76" s="5" t="inlineStr">
+        <is>
+          <t>Director of Supply Chain</t>
+        </is>
+      </c>
+      <c r="F76" s="5" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G76" s="5" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="7" t="inlineStr">
+        <is>
+          <t>Schur Technology A/S (Schur Group)</t>
+        </is>
+      </c>
+      <c r="B77" s="7" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="C77" s="7" t="inlineStr">
+        <is>
+          <t>Michael</t>
+        </is>
+      </c>
+      <c r="D77" s="7" t="inlineStr">
+        <is>
+          <t>Tr***n</t>
+        </is>
+      </c>
+      <c r="E77" s="7" t="inlineStr">
+        <is>
+          <t>Produktions Leder</t>
+        </is>
+      </c>
+      <c r="F77" s="7" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G77" s="7" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="5" t="inlineStr">
+        <is>
+          <t>Aasted ApS</t>
+        </is>
+      </c>
+      <c r="B78" s="5" t="inlineStr">
+        <is>
+          <t>CEO/MD</t>
+        </is>
+      </c>
+      <c r="C78" s="5" t="inlineStr">
+        <is>
+          <t>Piet</t>
+        </is>
+      </c>
+      <c r="D78" s="5" t="inlineStr">
+        <is>
+          <t>Ta***n</t>
+        </is>
+      </c>
+      <c r="E78" s="5" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="F78" s="5" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G78" s="5" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="7" t="inlineStr">
+        <is>
+          <t>Aasted ApS</t>
+        </is>
+      </c>
+      <c r="B79" s="7" t="inlineStr">
+        <is>
+          <t>Technical Director/CTO</t>
+        </is>
+      </c>
+      <c r="C79" s="7" t="inlineStr">
+        <is>
+          <t>Henrik</t>
+        </is>
+      </c>
+      <c r="D79" s="7" t="inlineStr">
+        <is>
+          <t>He***n</t>
+        </is>
+      </c>
+      <c r="E79" s="7" t="inlineStr">
+        <is>
+          <t>Chief Technology Officer</t>
+        </is>
+      </c>
+      <c r="F79" s="7" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G79" s="7" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="5" t="inlineStr">
+        <is>
+          <t>Aasted ApS</t>
+        </is>
+      </c>
+      <c r="B80" s="5" t="inlineStr">
+        <is>
+          <t>Purchasing</t>
+        </is>
+      </c>
+      <c r="C80" s="5" t="inlineStr">
+        <is>
+          <t>Christian</t>
+        </is>
+      </c>
+      <c r="D80" s="5" t="inlineStr">
+        <is>
+          <t>Aa***d</t>
+        </is>
+      </c>
+      <c r="E80" s="5" t="inlineStr">
+        <is>
+          <t>Head of Purchasing Department</t>
+        </is>
+      </c>
+      <c r="F80" s="5" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G80" s="5" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="7" t="inlineStr">
+        <is>
+          <t>Aasted ApS</t>
+        </is>
+      </c>
+      <c r="B81" s="7" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="C81" s="7" t="inlineStr">
+        <is>
+          <t>Paw</t>
+        </is>
+      </c>
+      <c r="D81" s="7" t="inlineStr">
+        <is>
+          <t>Ne***l</t>
+        </is>
+      </c>
+      <c r="E81" s="7" t="inlineStr">
+        <is>
+          <t>Production Manager</t>
+        </is>
+      </c>
+      <c r="F81" s="7" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G81" s="7" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="5" t="inlineStr">
+        <is>
+          <t>Aasted ApS</t>
+        </is>
+      </c>
+      <c r="B82" s="5" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="C82" s="5" t="inlineStr">
+        <is>
+          <t>Niels</t>
+        </is>
+      </c>
+      <c r="D82" s="5" t="inlineStr">
+        <is>
+          <t>Ha***n</t>
+        </is>
+      </c>
+      <c r="E82" s="5" t="inlineStr">
+        <is>
+          <t>Head of Sales Engineering</t>
+        </is>
+      </c>
+      <c r="F82" s="5" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G82" s="5" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="7" t="inlineStr">
+        <is>
+          <t>Aasted ApS</t>
+        </is>
+      </c>
+      <c r="B83" s="7" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="C83" s="7" t="inlineStr">
+        <is>
+          <t>Allan</t>
+        </is>
+      </c>
+      <c r="D83" s="7" t="inlineStr">
+        <is>
+          <t>Aa***d</t>
+        </is>
+      </c>
+      <c r="E83" s="7" t="inlineStr">
+        <is>
+          <t>Vice Chairman, Owner</t>
+        </is>
+      </c>
+      <c r="F83" s="7" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G83" s="7" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="5" t="inlineStr">
+        <is>
+          <t>Varimixer A/S (Wodschow &amp; Co.)</t>
+        </is>
+      </c>
+      <c r="B84" s="5" t="inlineStr">
+        <is>
+          <t>CEO/MD</t>
+        </is>
+      </c>
+      <c r="C84" s="5" t="inlineStr">
+        <is>
+          <t>Paw</t>
+        </is>
+      </c>
+      <c r="D84" s="5" t="inlineStr">
+        <is>
+          <t>Soe</t>
+        </is>
+      </c>
+      <c r="E84" s="5" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="F84" s="5" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G84" s="5" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="7" t="inlineStr">
+        <is>
+          <t>Varimixer A/S (Wodschow &amp; Co.)</t>
+        </is>
+      </c>
+      <c r="B85" s="7" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="C85" s="7" t="inlineStr">
+        <is>
+          <t>Jesper</t>
+        </is>
+      </c>
+      <c r="D85" s="7" t="inlineStr">
+        <is>
+          <t>Ol***n</t>
+        </is>
+      </c>
+      <c r="E85" s="7" t="inlineStr">
+        <is>
+          <t>Production Manager</t>
+        </is>
+      </c>
+      <c r="F85" s="7" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G85" s="7" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="5" t="inlineStr">
+        <is>
+          <t>Chocoma ApS</t>
+        </is>
+      </c>
+      <c r="B86" s="5" t="inlineStr">
+        <is>
+          <t>CEO/MD (Owner)</t>
+        </is>
+      </c>
+      <c r="C86" s="5" t="inlineStr">
+        <is>
+          <t>Christian</t>
+        </is>
+      </c>
+      <c r="D86" s="5" t="inlineStr">
+        <is>
+          <t>Ni***n</t>
+        </is>
+      </c>
+      <c r="E86" s="5" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="F86" s="5" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G86" s="5" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="7" t="inlineStr">
+        <is>
+          <t>Sealing System 2024 A/S</t>
+        </is>
+      </c>
+      <c r="B87" s="7" t="inlineStr">
+        <is>
+          <t>CEO/MD</t>
+        </is>
+      </c>
+      <c r="C87" s="7" t="inlineStr">
+        <is>
+          <t>Ole</t>
+        </is>
+      </c>
+      <c r="D87" s="7" t="inlineStr">
+        <is>
+          <t>Je***n</t>
+        </is>
+      </c>
+      <c r="E87" s="7" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="F87" s="7" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G87" s="7" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="5" t="inlineStr">
+        <is>
+          <t>Sealing System 2024 A/S</t>
+        </is>
+      </c>
+      <c r="B88" s="5" t="inlineStr">
+        <is>
+          <t>Purchasing/Procurement</t>
+        </is>
+      </c>
+      <c r="C88" s="5" t="inlineStr">
+        <is>
+          <t>Dion</t>
+        </is>
+      </c>
+      <c r="D88" s="5" t="inlineStr">
+        <is>
+          <t>La***n</t>
+        </is>
+      </c>
+      <c r="E88" s="5" t="inlineStr">
+        <is>
+          <t>Procurement Manager</t>
+        </is>
+      </c>
+      <c r="F88" s="5" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G88" s="5" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="7" t="inlineStr">
+        <is>
+          <t>Sealing System 2024 A/S</t>
+        </is>
+      </c>
+      <c r="B89" s="7" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="C89" s="7" t="inlineStr">
+        <is>
+          <t>Tonny</t>
+        </is>
+      </c>
+      <c r="D89" s="7" t="inlineStr">
+        <is>
+          <t>Ra***k</t>
+        </is>
+      </c>
+      <c r="E89" s="7" t="inlineStr">
+        <is>
+          <t>Engineering Manager</t>
+        </is>
+      </c>
+      <c r="F89" s="7" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G89" s="7" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="5" t="inlineStr">
+        <is>
+          <t>Sealing System 2024 A/S</t>
+        </is>
+      </c>
+      <c r="B90" s="5" t="inlineStr">
+        <is>
+          <t>Technical Director</t>
+        </is>
+      </c>
+      <c r="C90" s="5" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="D90" s="5" t="inlineStr">
+        <is>
+          <t>Pe***n</t>
+        </is>
+      </c>
+      <c r="E90" s="5" t="inlineStr">
+        <is>
+          <t>Technical Director</t>
+        </is>
+      </c>
+      <c r="F90" s="5" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G90" s="5" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="7" t="inlineStr">
+        <is>
+          <t>Sealing System 2024 A/S</t>
+        </is>
+      </c>
+      <c r="B91" s="7" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="C91" s="7" t="inlineStr">
+        <is>
+          <t>Rasmus</t>
+        </is>
+      </c>
+      <c r="D91" s="7" t="inlineStr">
+        <is>
+          <t>Da***n</t>
+        </is>
+      </c>
+      <c r="E91" s="7" t="inlineStr">
+        <is>
+          <t>Manager of Electrical Engineering &amp; Manufacturing</t>
+        </is>
+      </c>
+      <c r="F91" s="7" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G91" s="7" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="5" t="inlineStr">
+        <is>
+          <t>Dansk Maskin Teknik A/S (DMT)</t>
+        </is>
+      </c>
+      <c r="B92" s="5" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="C92" s="5" t="inlineStr">
+        <is>
+          <t>Andreas</t>
+        </is>
+      </c>
+      <c r="D92" s="5" t="inlineStr">
+        <is>
+          <t>La***n</t>
+        </is>
+      </c>
+      <c r="E92" s="5" t="inlineStr">
+        <is>
+          <t>Head of Mechanical Engineering</t>
+        </is>
+      </c>
+      <c r="F92" s="5" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G92" s="5" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="7" t="inlineStr">
+        <is>
+          <t>Micro Matic A/S</t>
+        </is>
+      </c>
+      <c r="B93" s="7" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="C93" s="7" t="inlineStr">
+        <is>
+          <t>Thomas</t>
+        </is>
+      </c>
+      <c r="D93" s="7" t="inlineStr">
+        <is>
+          <t>Ma***g</t>
+        </is>
+      </c>
+      <c r="E93" s="7" t="inlineStr">
+        <is>
+          <t>Head of Engineering</t>
+        </is>
+      </c>
+      <c r="F93" s="7" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G93" s="7" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="5" t="inlineStr">
+        <is>
+          <t>Micro Matic A/S</t>
+        </is>
+      </c>
+      <c r="B94" s="5" t="inlineStr">
+        <is>
+          <t>Purchasing/Procurement</t>
+        </is>
+      </c>
+      <c r="C94" s="5" t="inlineStr">
+        <is>
+          <t>Danny</t>
+        </is>
+      </c>
+      <c r="D94" s="5" t="inlineStr">
+        <is>
+          <t>Li***e</t>
+        </is>
+      </c>
+      <c r="E94" s="5" t="inlineStr">
+        <is>
+          <t>Project Manager - Group Procurement</t>
+        </is>
+      </c>
+      <c r="F94" s="5" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G94" s="5" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="7" t="inlineStr">
+        <is>
+          <t>Micro Matic A/S</t>
+        </is>
+      </c>
+      <c r="B95" s="7" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="C95" s="7" t="inlineStr">
+        <is>
+          <t>Kristian</t>
+        </is>
+      </c>
+      <c r="D95" s="7" t="inlineStr">
+        <is>
+          <t>An***n</t>
+        </is>
+      </c>
+      <c r="E95" s="7" t="inlineStr">
+        <is>
+          <t>Production Manager</t>
+        </is>
+      </c>
+      <c r="F95" s="7" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G95" s="7" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="5" t="inlineStr">
+        <is>
+          <t>Flexmatic (now SteelXperts ApS)</t>
+        </is>
+      </c>
+      <c r="B96" s="5" t="inlineStr">
+        <is>
+          <t>CEO/MD</t>
+        </is>
+      </c>
+      <c r="C96" s="5" t="inlineStr">
+        <is>
+          <t>Bjarne</t>
+        </is>
+      </c>
+      <c r="D96" s="5" t="inlineStr">
+        <is>
+          <t>So***n</t>
+        </is>
+      </c>
+      <c r="E96" s="5" t="inlineStr">
+        <is>
+          <t>Adm. Direktor og Medejer</t>
+        </is>
+      </c>
+      <c r="F96" s="5" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G96" s="5" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="7" t="inlineStr">
+        <is>
+          <t>Dalum Beverage Equipment ApS</t>
+        </is>
+      </c>
+      <c r="B97" s="7" t="inlineStr">
+        <is>
+          <t>CEO/MD</t>
+        </is>
+      </c>
+      <c r="C97" s="7" t="inlineStr">
+        <is>
+          <t>Kim</t>
+        </is>
+      </c>
+      <c r="D97" s="7" t="inlineStr">
+        <is>
+          <t>Da***m</t>
+        </is>
+      </c>
+      <c r="E97" s="7" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="F97" s="7" t="inlineStr">
+        <is>
+          <t>Denmark</t>
+        </is>
+      </c>
+      <c r="G97" s="7" t="inlineStr">
+        <is>
+          <t>(enrich to reveal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="12" t="inlineStr">
+        <is>
+          <t>96 decision-makers across 36 of 49 companies, pulled via Apollo People Search (FREE, no credits).</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="13" t="inlineStr">
+        <is>
+          <t>Last names are MASKED by Apollo (e.g. Ra***n). Full name + business email + LinkedIn URL require an</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="13" t="inlineStr">
+        <is>
+          <t>enrichment pass (~1 lead credit per person). 13 companies returned no Apollo records: Kroma, BoPil, Trepko,</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="13" t="inlineStr">
+        <is>
+          <t>Landia, CTI Process, Attec (merged into Frontmatec), Butina, DanfoTech, Skals, Bila, Haas-Meincke, Bruel, FH Scandinox.</t>
         </is>
       </c>
     </row>
@@ -9289,7 +12507,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="inlineStr">
+      <c r="A10" s="13" t="inlineStr">
         <is>
           <t>All supplier assignments in this workbook are INFERRED (no public BOM). Verify per account before outreach.</t>
         </is>

</xml_diff>

<commit_message>
Enrich full Apollo roster (94 contacts, verified emails + LinkedIn) into Batch 1 Excel
</commit_message>
<xml_diff>
--- a/market-research/I-MAK_Denmark_Batch1_Food.xlsx
+++ b/market-research/I-MAK_Denmark_Batch1_Food.xlsx
@@ -131,7 +131,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -158,6 +158,15 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -8681,16 +8690,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G102"/>
+  <dimension ref="A1:H99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="46" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8701,32 +8711,37 @@
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>Role Category</t>
+          <t>Role</t>
         </is>
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
-          <t>First Name</t>
+          <t>Full Name</t>
         </is>
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
-          <t>Last Name (masked)</t>
+          <t>Title</t>
         </is>
       </c>
       <c r="E1" s="4" t="inlineStr">
         <is>
-          <t>Exact Title</t>
+          <t>Business Email</t>
         </is>
       </c>
       <c r="F1" s="4" t="inlineStr">
         <is>
+          <t>Email Status</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>LinkedIn URL</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
           <t>Location</t>
-        </is>
-      </c>
-      <c r="G1" s="4" t="inlineStr">
-        <is>
-          <t>Full Name / Email / LinkedIn</t>
         </is>
       </c>
     </row>
@@ -8743,27 +8758,32 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>Dirk</t>
+          <t>Dirk Haemling</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>Ha***g</t>
+          <t>CEO Gram-Equipment A/S</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>CEO Gram-Equipment A/S</t>
-        </is>
-      </c>
-      <c r="F2" s="5" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>dh@gram-equipment.com</t>
+        </is>
+      </c>
+      <c r="F2" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/dirk-haemling-29ba3845</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>Hamburg, Germany</t>
         </is>
       </c>
     </row>
@@ -8775,32 +8795,37 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>Purchasing/Procurement</t>
+          <t>Purchasing</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>Peter</t>
+          <t>Peter Rasmussen</t>
         </is>
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>Ra***n</t>
+          <t>Strategic Procurement Manager &amp; Lead</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>Strategic Procurement Manager &amp; Lead</t>
-        </is>
-      </c>
-      <c r="F3" s="7" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>pera@gram-equipment.com</t>
+        </is>
+      </c>
+      <c r="F3" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G3" s="7" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/peter-lilholm-rasmussen-71578511</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>Fredericia, DK</t>
         </is>
       </c>
     </row>
@@ -8817,27 +8842,32 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>Michael</t>
+          <t>Michael Cornelius</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Co***s</t>
+          <t>R&amp;D Manager</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>R&amp;D Manager</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>mic@gram-equipment.com</t>
+        </is>
+      </c>
+      <c r="F4" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/michael-cornelius-47529b54</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>S. Denmark</t>
         </is>
       </c>
     </row>
@@ -8854,27 +8884,32 @@
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>Jens</t>
+          <t>Jens Hansen</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>Ha***n</t>
+          <t>Production Manager</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>Production Manager</t>
-        </is>
-      </c>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>jph@gram-equipment.com</t>
+        </is>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/jens-peder-hansen-b5217571</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>Central DK</t>
         </is>
       </c>
     </row>
@@ -8891,27 +8926,32 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Jan</t>
+          <t>Jan Hansen</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Ha***n</t>
+          <t>CFO, Co-owner</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>CFO, Co-owner</t>
-        </is>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>jhh@cabinplant.com</t>
+        </is>
+      </c>
+      <c r="F6" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/jan-helskov-hansen-9491b06</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>S. Denmark</t>
         </is>
       </c>
     </row>
@@ -8923,32 +8963,37 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Purchasing/Procurement</t>
+          <t>Purchasing</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Juergen</t>
+          <t>Juergen Juergensen</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>Ju***n</t>
+          <t>Procurement Manager</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>Procurement Manager</t>
-        </is>
-      </c>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>jju@cabinplant.com</t>
+        </is>
+      </c>
+      <c r="F7" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/jürgen-jürgensen-68940618</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>Haarby, DK</t>
         </is>
       </c>
     </row>
@@ -8965,27 +9010,32 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Michael</t>
+          <t>Michael Pedersen</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Pe***n</t>
+          <t>Engineering Manager - Processing</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>Engineering Manager - Processing</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>mpe@cabinplant.com</t>
+        </is>
+      </c>
+      <c r="F8" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/michael-krog-pedersen-22376789</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>S. Denmark</t>
         </is>
       </c>
     </row>
@@ -9002,34 +9052,39 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Henrik</t>
+          <t>Henrik Sondergaard</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>So***d</t>
+          <t>Production Manager</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>Production Manager</t>
-        </is>
-      </c>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>hsj@cabinplant.com</t>
+        </is>
+      </c>
+      <c r="F9" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/henrik-søndergaard-91b272114</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>S. Denmark</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Carsoe (Carsoe Group A/S)</t>
+          <t>Carsoe / KM Fish Machinery</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
@@ -9039,34 +9094,35 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Soren</t>
+          <t>Soren Klyvo</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Kl***o</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
           <t>CEO</t>
         </is>
       </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+      <c r="E10" s="5" t="inlineStr"/>
+      <c r="F10" s="13" t="inlineStr">
+        <is>
+          <t>unavailable</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/klyvo</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>N. Denmark</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>Carsoe (Carsoe Group A/S)</t>
+          <t>Carsoe / KM Fish Machinery</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
@@ -9076,71 +9132,81 @@
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Henrik</t>
+          <t>Henrik Poulsen</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>Po***n</t>
+          <t>CTO</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>CTO</t>
-        </is>
-      </c>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>hjp@carsoe.com</t>
+        </is>
+      </c>
+      <c r="F11" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/henrik-poulsen-38aa5416</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Aarhus, DK</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Carsoe (Carsoe Group A/S)</t>
+          <t>Carsoe / KM Fish Machinery</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Purchasing/Procurement</t>
+          <t>Purchasing</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>Doris</t>
+          <t>Doris Hamann</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Ha***n</t>
+          <t>Procurement &amp; Logistics Manager</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>Procurement &amp; Logistics Manager</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>dha@carsoe.com</t>
+        </is>
+      </c>
+      <c r="F12" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/doris-hamann-43178726</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>Aalborg, DK</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>Carsoe (Carsoe Group A/S)</t>
+          <t>Carsoe / KM Fish Machinery</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
@@ -9150,330 +9216,355 @@
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Magnus</t>
+          <t>Magnus Heegaard</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>He***d</t>
-        </is>
-      </c>
-      <c r="E13" s="7" t="inlineStr">
-        <is>
           <t>Manager of Mechanical Engineering</t>
         </is>
       </c>
-      <c r="F13" s="7" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+      <c r="E13" s="7" t="inlineStr"/>
+      <c r="F13" s="13" t="inlineStr">
+        <is>
+          <t>unavailable</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/magnus-heegaard-5318b848</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>Aalborg, DK</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>KM Fish Machinery A/S</t>
+          <t>Uni-Food Technic A/S</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>CEO/MD</t>
+          <t>CEO/MD (Owner)</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Soren</t>
+          <t>Jeppe Christensen</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Kl***o</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>CEO (shared Carsoe org)</t>
-        </is>
-      </c>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>Chief Executive Officer, Owner</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr"/>
+      <c r="F14" s="13" t="inlineStr">
+        <is>
+          <t>unavailable</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/jeppe-christensen-4823b933</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>Aalborg, DK</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>KM Fish Machinery A/S</t>
+          <t>Uni-Food Technic A/S</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Purchasing/Procurement</t>
+          <t>Production</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Doris</t>
+          <t>Michael Hansen</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>Ha***n</t>
-        </is>
-      </c>
-      <c r="E15" s="7" t="inlineStr">
-        <is>
-          <t>Procurement &amp; Logistics Manager (shared Carsoe org)</t>
-        </is>
-      </c>
-      <c r="F15" s="7" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>Production Manager</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr"/>
+      <c r="F15" s="13" t="inlineStr">
+        <is>
+          <t>unavailable</t>
         </is>
       </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/michael-mandrup-hansen-65a68b107</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>Storvorde, DK</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Uni-Food Technic A/S</t>
+          <t>Kaj Olesen A/S</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>CEO/MD (Owner)</t>
+          <t>CEO/MD</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Jeppe</t>
+          <t>Jacob Olesen</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Ch***n</t>
+          <t>CEO</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>Chief Executive Officer, Owner</t>
-        </is>
-      </c>
-      <c r="F16" s="5" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>jo@kajolesen.dk</t>
+        </is>
+      </c>
+      <c r="F16" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/jacob-olesen-2838ab141</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>S. Denmark</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>Uni-Food Technic A/S</t>
+          <t>IRAS A/S</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Production</t>
+          <t>CEO/MD (Owner)</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>Michael</t>
+          <t>Peter Rasmussen</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>Ha***n</t>
+          <t>Owner (CEO &amp; Owner)</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>Production Manager</t>
-        </is>
-      </c>
-      <c r="F17" s="7" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>psr@iras.dk</t>
+        </is>
+      </c>
+      <c r="F17" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/peter-s-rasmussen-2b98b91a2</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>S. Denmark</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Kaj Olesen A/S</t>
+          <t>DSI Freezing Solutions / DSI Dantech A/S</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>CEO/MD</t>
+          <t>Supply Chain</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Jacob</t>
+          <t>Hans Viggaard</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Ol***n</t>
+          <t>Supply Chain Director (interim)</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>CEO</t>
-        </is>
-      </c>
-      <c r="F18" s="5" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>hans.viggaard@dsidantech.com</t>
+        </is>
+      </c>
+      <c r="F18" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/viggaard</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>Aarhus, DK</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>IRAS A/S</t>
+          <t>DSI Freezing Solutions / DSI Dantech A/S</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>CEO/MD (Owner)</t>
+          <t>Production</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>Peter</t>
+          <t>Anders Christensen</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>Ra***n</t>
+          <t>Production Manager</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>Owner</t>
-        </is>
-      </c>
-      <c r="F19" s="7" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>anders.christensen@dsidantech.com</t>
+        </is>
+      </c>
+      <c r="F19" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/anders-christensen-4b847610</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>Saeby, DK</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>DSI Freezing Solutions / DSI Dantech A/S</t>
+          <t>Qupaq A/S</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Supply Chain</t>
+          <t>CEO/MD</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>Hans</t>
+          <t>Christian Bols</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Vi***d</t>
-        </is>
-      </c>
-      <c r="E20" s="5" t="inlineStr">
-        <is>
-          <t>Supply Chain Director (interim)</t>
-        </is>
-      </c>
-      <c r="F20" s="5" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>Chief Executive Officer</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr"/>
+      <c r="F20" s="13" t="inlineStr">
+        <is>
+          <t>unavailable</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/christian-bols-16aa9433</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>Aalborg, DK</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>DSI Freezing Solutions / DSI Dantech A/S</t>
+          <t>Globaq Solutions (ex-Billund Aquaculture)</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Production</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>Anders</t>
+          <t>Carlos Ardissoni</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>Ch***n</t>
-        </is>
-      </c>
-      <c r="E21" s="7" t="inlineStr">
-        <is>
-          <t>Production Manager</t>
-        </is>
-      </c>
-      <c r="F21" s="7" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>Engineering Manager</t>
+        </is>
+      </c>
+      <c r="E21" s="7" t="inlineStr"/>
+      <c r="F21" s="13" t="inlineStr">
+        <is>
+          <t>unavailable</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/carlos-ardissoni-811a617</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>Billund, DK</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>Qupaq A/S</t>
+          <t>Primodan A/S</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
@@ -9483,71 +9574,77 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Christian</t>
+          <t>Lars Henriksen</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Bo***s</t>
+          <t>CEO</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>Chief Executive Officer</t>
-        </is>
-      </c>
-      <c r="F22" s="5" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>lh@primodan.com</t>
+        </is>
+      </c>
+      <c r="F22" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/lars-henriksen-4ab07723</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>Zealand, DK</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>Globaq Solutions (ex-Billund Aquaculture)</t>
+          <t>Primodan A/S</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>Production</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>Carlos</t>
+          <t>Tommy Olsen</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>Ar***i</t>
-        </is>
-      </c>
-      <c r="E23" s="7" t="inlineStr">
-        <is>
-          <t>Engineering Manager</t>
-        </is>
-      </c>
-      <c r="F23" s="7" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>Production Manager</t>
+        </is>
+      </c>
+      <c r="E23" s="7" t="inlineStr"/>
+      <c r="F23" s="13" t="inlineStr">
+        <is>
+          <t>unavailable</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/tommy-olsen-67ba4b100</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>Bjæverskov, DK</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Primodan A/S</t>
+          <t>SiccaDania A/S</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
@@ -9557,108 +9654,119 @@
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Lars</t>
+          <t>Lone Hogholt</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>He***n</t>
+          <t>CEO SiccaDania Holding</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t>CEO</t>
-        </is>
-      </c>
-      <c r="F24" s="5" t="inlineStr">
+          <t>lone.hoegholt@siccadania.com</t>
+        </is>
+      </c>
+      <c r="F24" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/lonehoegholt</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
         <is>
           <t>Denmark</t>
-        </is>
-      </c>
-      <c r="G24" s="5" t="inlineStr">
-        <is>
-          <t>(enrich to reveal)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>Primodan A/S</t>
+          <t>SiccaDania A/S</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Production</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>Tommy</t>
+          <t>Willy Matyjasik</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>Ol***n</t>
-        </is>
-      </c>
-      <c r="E25" s="7" t="inlineStr">
-        <is>
-          <t>Production Manager</t>
-        </is>
-      </c>
-      <c r="F25" s="7" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>Engineering Manager</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr"/>
+      <c r="F25" s="13" t="inlineStr">
+        <is>
+          <t>unavailable</t>
         </is>
       </c>
       <c r="G25" s="7" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/willy-matyjasik-b3a7a6163</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
+        <is>
+          <t>Jyllinge, DK</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>SiccaDania A/S</t>
+          <t>Tetra Pak Hoyer A/S</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>CEO/MD</t>
+          <t>Production</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Lone</t>
+          <t>Lasse Jensen</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Ho***t</t>
+          <t>Production Manager</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>CEO SiccaDania Holding</t>
-        </is>
-      </c>
-      <c r="F26" s="5" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>lasse.jensen@tetrapak.com</t>
+        </is>
+      </c>
+      <c r="F26" s="14" t="inlineStr">
+        <is>
+          <t>extrapolated</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/lasse-bach-jensen-71478015b</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>Aalborg, DK</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>SiccaDania A/S</t>
+          <t>Tetra Pak Hoyer A/S</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
@@ -9668,27 +9776,28 @@
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>Willy</t>
+          <t>Morten Ostli</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>Ma***k</t>
-        </is>
-      </c>
-      <c r="E27" s="7" t="inlineStr">
-        <is>
           <t>Engineering Manager</t>
         </is>
       </c>
-      <c r="F27" s="7" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+      <c r="E27" s="7" t="inlineStr"/>
+      <c r="F27" s="13" t="inlineStr">
+        <is>
+          <t>unavailable</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/morten-emil-østli</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>Aarhus, DK</t>
         </is>
       </c>
     </row>
@@ -9700,32 +9809,37 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Production</t>
+          <t>Purchasing</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Lasse</t>
+          <t>Allen Levy</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Je***n</t>
+          <t>Senior Innovation Procurement Manager</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>Production Manager</t>
-        </is>
-      </c>
-      <c r="F28" s="5" t="inlineStr">
+          <t>allen.levy@tetrapak.com</t>
+        </is>
+      </c>
+      <c r="F28" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/allen-levy</t>
+        </is>
+      </c>
+      <c r="H28" s="5" t="inlineStr">
         <is>
           <t>Denmark</t>
-        </is>
-      </c>
-      <c r="G28" s="5" t="inlineStr">
-        <is>
-          <t>(enrich to reveal)</t>
         </is>
       </c>
     </row>
@@ -9737,32 +9851,37 @@
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>R&amp;D</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>Morten</t>
+          <t>Soren Andersen</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>Os***i</t>
+          <t>R&amp;D Project Manager</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>Engineering Manager</t>
-        </is>
-      </c>
-      <c r="F29" s="7" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>soren.andersen@tetrapak.com</t>
+        </is>
+      </c>
+      <c r="F29" s="14" t="inlineStr">
+        <is>
+          <t>extrapolated</t>
         </is>
       </c>
       <c r="G29" s="7" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/søren-andersen-75279118</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>N. Denmark</t>
         </is>
       </c>
     </row>
@@ -9774,32 +9893,37 @@
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>Purchasing/Procurement</t>
+          <t>Supply Chain</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>Allen</t>
+          <t>Bente Damgaard</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>Le***y</t>
+          <t>Supply Manager</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>Senior Innovation Procurement Manager</t>
-        </is>
-      </c>
-      <c r="F30" s="5" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>bente.damgaard@tetrapak.com</t>
+        </is>
+      </c>
+      <c r="F30" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/bente-damgaard-8202048</t>
+        </is>
+      </c>
+      <c r="H30" s="5" t="inlineStr">
+        <is>
+          <t>Aarhus, DK</t>
         </is>
       </c>
     </row>
@@ -9811,76 +9935,82 @@
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>R&amp;D</t>
+          <t>Technical Director</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>Soren</t>
+          <t>Steen Rasmussen</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>An***n</t>
-        </is>
-      </c>
-      <c r="E31" s="7" t="inlineStr">
-        <is>
-          <t>R&amp;D Project Manager</t>
-        </is>
-      </c>
-      <c r="F31" s="7" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>Technical Sales Director</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="inlineStr"/>
+      <c r="F31" s="13" t="inlineStr">
+        <is>
+          <t>unavailable</t>
         </is>
       </c>
       <c r="G31" s="7" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/rasmussen-steen-a933a56</t>
+        </is>
+      </c>
+      <c r="H31" s="7" t="inlineStr">
+        <is>
+          <t>Central DK</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>Tetra Pak Hoyer A/S</t>
+          <t>GEA Process Engineering A/S (ex-Niro)</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>Supply Chain</t>
+          <t>CEO/MD</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>Bente</t>
+          <t>Claus Thorsen</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>Da***d</t>
+          <t>Country Mgr Dir DACH &amp; Nordics NPE / MD GEA Liquid Technologies</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>Supply Manager</t>
-        </is>
-      </c>
-      <c r="F32" s="5" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>claus.thorsen@gea.com</t>
+        </is>
+      </c>
+      <c r="F32" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/claus-thorsen-7b7b2030</t>
+        </is>
+      </c>
+      <c r="H32" s="5" t="inlineStr">
+        <is>
+          <t>Silkeborg, DK</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>Tetra Pak Hoyer A/S</t>
+          <t>GEA Process Engineering A/S (ex-Niro)</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
@@ -9890,27 +10020,28 @@
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>(Mr.)</t>
+          <t>Poul-Erik Aagaard</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>Ra***n</t>
-        </is>
-      </c>
-      <c r="E33" s="7" t="inlineStr">
-        <is>
-          <t>Technical Sales Director</t>
-        </is>
-      </c>
-      <c r="F33" s="7" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>Technical Director</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr"/>
+      <c r="F33" s="13" t="inlineStr">
+        <is>
+          <t>unavailable</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/poul-erik-aagaard-9a50308b</t>
+        </is>
+      </c>
+      <c r="H33" s="7" t="inlineStr">
+        <is>
+          <t>Central DK</t>
         </is>
       </c>
     </row>
@@ -9922,32 +10053,33 @@
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>CEO/MD</t>
+          <t>R&amp;D</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>Claus</t>
+          <t>Anders Reske-Nielsen</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>Th***n</t>
-        </is>
-      </c>
-      <c r="E34" s="5" t="inlineStr">
-        <is>
-          <t>Country Mgr Dir DACH &amp; Nordics NPE / MD GEA Liquid Technologies A/S</t>
-        </is>
-      </c>
-      <c r="F34" s="5" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>Head of Digitalization and Automation R&amp;D</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr"/>
+      <c r="F34" s="13" t="inlineStr">
+        <is>
+          <t>unavailable</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/andersreske</t>
+        </is>
+      </c>
+      <c r="H34" s="5" t="inlineStr">
+        <is>
+          <t>Copenhagen, DK</t>
         </is>
       </c>
     </row>
@@ -9959,32 +10091,37 @@
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>Technical Director</t>
+          <t>Supply Chain</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>Poul-Erik</t>
+          <t>Lars Holm-Pedersen</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>Aa***d</t>
+          <t>Senior Director Procurement &amp; Supply Chain</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>Technical Director</t>
-        </is>
-      </c>
-      <c r="F35" s="7" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>lars.holm-pedersen@gea.com</t>
+        </is>
+      </c>
+      <c r="F35" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G35" s="7" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/larsholm-pedersen</t>
+        </is>
+      </c>
+      <c r="H35" s="7" t="inlineStr">
+        <is>
+          <t>Copenhagen, DK</t>
         </is>
       </c>
     </row>
@@ -9996,32 +10133,37 @@
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>R&amp;D</t>
+          <t>Purchasing</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>Anders</t>
+          <t>Rene Clausen</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>Re***n</t>
+          <t>Head of Procurement (interim), GEA Liquid Technology</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>Head of Digitalization and Automation R&amp;D</t>
-        </is>
-      </c>
-      <c r="F36" s="5" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>rene.clausen@gea.com</t>
+        </is>
+      </c>
+      <c r="F36" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/rené-clausen-0a716936</t>
+        </is>
+      </c>
+      <c r="H36" s="5" t="inlineStr">
+        <is>
+          <t>Copenhagen, DK</t>
         </is>
       </c>
     </row>
@@ -10033,298 +10175,330 @@
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>Supply Chain</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>Lars</t>
+          <t>Peter Plett</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>Ho***n</t>
+          <t>Head of Project Engineering - Membrane Filtration</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>Senior Director Procurement &amp; Supply Chain</t>
-        </is>
-      </c>
-      <c r="F37" s="7" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>peter.plett@gea.com</t>
+        </is>
+      </c>
+      <c r="F37" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/peter-plett-49837935</t>
+        </is>
+      </c>
+      <c r="H37" s="7" t="inlineStr">
+        <is>
+          <t>Skanderborg, DK</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>GEA Process Engineering A/S (ex-Niro)</t>
+          <t>SPX FLOW Danmark (APV)</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>Purchasing/Procurement</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>Rene</t>
+          <t>Lis Rasmussen</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>Cl***n</t>
-        </is>
-      </c>
-      <c r="E38" s="5" t="inlineStr">
-        <is>
-          <t>Head of Procurement (interim), GEA Liquid Technology A/S</t>
-        </is>
-      </c>
-      <c r="F38" s="5" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>Engineering Manager, Process Technology Membrane &amp; UHT</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr"/>
+      <c r="F38" s="13" t="inlineStr">
+        <is>
+          <t>unavailable</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/lis-fleng-rasmussen-b3719a6</t>
+        </is>
+      </c>
+      <c r="H38" s="5" t="inlineStr">
+        <is>
+          <t>Middelfart, DK</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
         <is>
-          <t>GEA Process Engineering A/S (ex-Niro)</t>
+          <t>NDT - Nordic Dairy Technology ApS</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>CEO/MD</t>
         </is>
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>Peter</t>
+          <t>Stig Petersen</t>
         </is>
       </c>
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>Pl***t</t>
-        </is>
-      </c>
-      <c r="E39" s="7" t="inlineStr">
-        <is>
-          <t>Head of Project Engineering - Membrane Filtration</t>
-        </is>
-      </c>
-      <c r="F39" s="7" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>Chief Executive Officer</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr"/>
+      <c r="F39" s="13" t="inlineStr">
+        <is>
+          <t>unavailable</t>
         </is>
       </c>
       <c r="G39" s="7" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/stig-victor-petersen-73754415</t>
+        </is>
+      </c>
+      <c r="H39" s="7" t="inlineStr">
+        <is>
+          <t>Aarhus, DK</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>SPX FLOW Danmark (APV)</t>
+          <t>Egatec A/S</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>CEO/MD</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>Lis</t>
+          <t>Rene Moller</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>Ra***n</t>
+          <t>Adm. Direktør / CEO</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>Engineering Manager, Process Technology Membrane &amp; UHT</t>
-        </is>
-      </c>
-      <c r="F40" s="5" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>rkm@egatec.dk</t>
+        </is>
+      </c>
+      <c r="F40" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/rené-kemp-møller-a0bbb644</t>
+        </is>
+      </c>
+      <c r="H40" s="5" t="inlineStr">
+        <is>
+          <t>S. Denmark</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
         <is>
-          <t>NDT - Nordic Dairy Technology ApS</t>
+          <t>Egatec A/S</t>
         </is>
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>CEO/MD</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
-          <t>Stig</t>
+          <t>Tommy Pedersen</t>
         </is>
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>Pe***n</t>
+          <t>Head of Engineering, Automation</t>
         </is>
       </c>
       <c r="E41" s="7" t="inlineStr">
         <is>
-          <t>Chief Executive Officer</t>
-        </is>
-      </c>
-      <c r="F41" s="7" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>ttp@egatec.dk</t>
+        </is>
+      </c>
+      <c r="F41" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G41" s="7" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/tommy-tjørnelund-pedersen-3692bb34</t>
+        </is>
+      </c>
+      <c r="H41" s="7" t="inlineStr">
+        <is>
+          <t>Odense, DK</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>Egatec A/S</t>
+          <t>Frontmatec Group</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>CEO/MD</t>
+          <t>Supply Chain</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>Rene</t>
+          <t>Thorbjorn Bentzen</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>Mo***r</t>
+          <t>Senior Director Supply Chain Europe</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
         <is>
-          <t>Adm. Direktor / CEO</t>
-        </is>
-      </c>
-      <c r="F42" s="5" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>thben@frontmatec.com</t>
+        </is>
+      </c>
+      <c r="F42" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/thorbjørn-bentzen-91a6231</t>
+        </is>
+      </c>
+      <c r="H42" s="5" t="inlineStr">
+        <is>
+          <t>Horsens, DK</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
         <is>
-          <t>Egatec A/S</t>
+          <t>Frontmatec Group</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>R&amp;D</t>
         </is>
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>Tommy</t>
+          <t>Thomas Lauridsen</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>Pe***n</t>
+          <t>R&amp;D Manager, Instruments</t>
         </is>
       </c>
       <c r="E43" s="7" t="inlineStr">
         <is>
-          <t>Head of Engineering, Automation</t>
-        </is>
-      </c>
-      <c r="F43" s="7" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>tla@frontmatec.com</t>
+        </is>
+      </c>
+      <c r="F43" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G43" s="7" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/thomas-lauridsen-8584b32</t>
+        </is>
+      </c>
+      <c r="H43" s="7" t="inlineStr">
+        <is>
+          <t>Slagelse, DK</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
         <is>
-          <t>Frontmatec Group</t>
+          <t>Scansteel foodtech A/S</t>
         </is>
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>Supply Chain</t>
+          <t>CEO/MD</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>Thorbjorn</t>
+          <t>Henrik Sandberg</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>Be***n</t>
+          <t>CEO/Owner</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t>Senior Director Supply Chain Europe</t>
-        </is>
-      </c>
-      <c r="F44" s="5" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>henrik.sandberg@scansteelfoodtech.com</t>
+        </is>
+      </c>
+      <c r="F44" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G44" s="5" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/henrik-sandberg-51617431</t>
+        </is>
+      </c>
+      <c r="H44" s="5" t="inlineStr">
+        <is>
+          <t>Zealand, DK</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
         <is>
-          <t>Frontmatec Group</t>
+          <t>Scansteel foodtech A/S</t>
         </is>
       </c>
       <c r="B45" s="7" t="inlineStr">
@@ -10334,27 +10508,32 @@
       </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Henrik Larsen</t>
         </is>
       </c>
       <c r="D45" s="7" t="inlineStr">
         <is>
-          <t>La***n</t>
+          <t>Project and R&amp;D Manager</t>
         </is>
       </c>
       <c r="E45" s="7" t="inlineStr">
         <is>
-          <t>R&amp;D Manager, Instruments</t>
-        </is>
-      </c>
-      <c r="F45" s="7" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>henrik.larsen@scansteelfoodtech.com</t>
+        </is>
+      </c>
+      <c r="F45" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G45" s="7" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/henrik-v-larsen-30b28329</t>
+        </is>
+      </c>
+      <c r="H45" s="7" t="inlineStr">
+        <is>
+          <t>Zealand, DK</t>
         </is>
       </c>
     </row>
@@ -10366,106 +10545,121 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>CEO/MD</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
         <is>
-          <t>Henrik</t>
+          <t>Mohammad Safdary</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>Sa***g</t>
+          <t>Technical Engineering Manager</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t>CEO/Owner</t>
-        </is>
-      </c>
-      <c r="F46" s="5" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>mohammad.safdary@scansteelfoodtech.com</t>
+        </is>
+      </c>
+      <c r="F46" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G46" s="5" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/mohammad-safdary-90a9ab115</t>
+        </is>
+      </c>
+      <c r="H46" s="5" t="inlineStr">
+        <is>
+          <t>Zealand, DK</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
         <is>
-          <t>Scansteel foodtech A/S</t>
+          <t>Fomaco A/S</t>
         </is>
       </c>
       <c r="B47" s="7" t="inlineStr">
         <is>
-          <t>R&amp;D</t>
+          <t>CEO/MD</t>
         </is>
       </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
-          <t>Henrik</t>
+          <t>Sebastian Mueller</t>
         </is>
       </c>
       <c r="D47" s="7" t="inlineStr">
         <is>
-          <t>La***n</t>
+          <t>CEO</t>
         </is>
       </c>
       <c r="E47" s="7" t="inlineStr">
         <is>
-          <t>Project and R&amp;D Manager</t>
-        </is>
-      </c>
-      <c r="F47" s="7" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>s.muller@fomaco.com</t>
+        </is>
+      </c>
+      <c r="F47" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G47" s="7" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/sebastian-müller-1147a0128</t>
+        </is>
+      </c>
+      <c r="H47" s="7" t="inlineStr">
+        <is>
+          <t>Zealand, DK</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>Scansteel foodtech A/S</t>
+          <t>Fomaco A/S</t>
         </is>
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>Technical Director</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>Mohammad</t>
+          <t>Carsten Giesel</t>
         </is>
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>Sa***y</t>
+          <t>CTO</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t>Technical Engineering Manager</t>
-        </is>
-      </c>
-      <c r="F48" s="5" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>c.giesel@fomaco.com</t>
+        </is>
+      </c>
+      <c r="F48" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G48" s="5" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/carstengiesel</t>
+        </is>
+      </c>
+      <c r="H48" s="5" t="inlineStr">
+        <is>
+          <t>Copenhagen, DK</t>
         </is>
       </c>
     </row>
@@ -10477,76 +10671,82 @@
       </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>CEO/MD</t>
+          <t>Production</t>
         </is>
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>Sebastian</t>
+          <t>Ole Nielsen</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr">
         <is>
-          <t>Mu***r</t>
-        </is>
-      </c>
-      <c r="E49" s="7" t="inlineStr">
-        <is>
-          <t>CEO</t>
-        </is>
-      </c>
-      <c r="F49" s="7" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>Production Manager</t>
+        </is>
+      </c>
+      <c r="E49" s="7" t="inlineStr"/>
+      <c r="F49" s="13" t="inlineStr">
+        <is>
+          <t>unavailable</t>
         </is>
       </c>
       <c r="G49" s="7" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/ole-nielsen-b5a08b111</t>
+        </is>
+      </c>
+      <c r="H49" s="7" t="inlineStr">
+        <is>
+          <t>Zealand, DK</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>Fomaco A/S</t>
+          <t>JS Proputec A/S</t>
         </is>
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>Technical Director</t>
+          <t>CEO/MD</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>Carsten</t>
+          <t>Morten Brandborg</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>Gi***l</t>
+          <t>Chief Executive Officer</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
         <is>
-          <t>CTO</t>
-        </is>
-      </c>
-      <c r="F50" s="5" t="inlineStr">
+          <t>mbr@jsproputec.com</t>
+        </is>
+      </c>
+      <c r="F50" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="G50" s="5" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/morten-brandborg-9ab7ab12</t>
+        </is>
+      </c>
+      <c r="H50" s="5" t="inlineStr">
         <is>
           <t>Denmark</t>
-        </is>
-      </c>
-      <c r="G50" s="5" t="inlineStr">
-        <is>
-          <t>(enrich to reveal)</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
         <is>
-          <t>Fomaco A/S</t>
+          <t>JS Proputec A/S</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
@@ -10556,34 +10756,35 @@
       </c>
       <c r="C51" s="7" t="inlineStr">
         <is>
-          <t>Ole</t>
+          <t>Bjarne Jensen</t>
         </is>
       </c>
       <c r="D51" s="7" t="inlineStr">
         <is>
-          <t>Ni***n</t>
-        </is>
-      </c>
-      <c r="E51" s="7" t="inlineStr">
-        <is>
           <t>Production Manager</t>
         </is>
       </c>
-      <c r="F51" s="7" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+      <c r="E51" s="7" t="inlineStr"/>
+      <c r="F51" s="13" t="inlineStr">
+        <is>
+          <t>unavailable</t>
         </is>
       </c>
       <c r="G51" s="7" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/bjarne-søren-jensen-53a7345</t>
+        </is>
+      </c>
+      <c r="H51" s="7" t="inlineStr">
+        <is>
+          <t>N. Denmark</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>JS Proputec A/S</t>
+          <t>BAADER Food Systems Denmark A/S (ex-LINCO)</t>
         </is>
       </c>
       <c r="B52" s="5" t="inlineStr">
@@ -10593,64 +10794,74 @@
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>Morten</t>
+          <t>Henning Pedersen</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>Br***g</t>
+          <t>Managing Director / CEO</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t>Chief Executive Officer</t>
-        </is>
-      </c>
-      <c r="F52" s="5" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>henning.pedersen@baader.com</t>
+        </is>
+      </c>
+      <c r="F52" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G52" s="5" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/henning-b-pedersen-258152a2</t>
+        </is>
+      </c>
+      <c r="H52" s="5" t="inlineStr">
+        <is>
+          <t>Central DK</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
         <is>
-          <t>JS Proputec A/S</t>
+          <t>BAADER Food Systems Denmark A/S (ex-LINCO)</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>Production</t>
+          <t>R&amp;D</t>
         </is>
       </c>
       <c r="C53" s="7" t="inlineStr">
         <is>
-          <t>Bjarne</t>
+          <t>Michael Hansen</t>
         </is>
       </c>
       <c r="D53" s="7" t="inlineStr">
         <is>
-          <t>Je***n</t>
+          <t>Head of R&amp;D</t>
         </is>
       </c>
       <c r="E53" s="7" t="inlineStr">
         <is>
-          <t>Production Manager</t>
-        </is>
-      </c>
-      <c r="F53" s="7" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>michael.hansen@baader.com</t>
+        </is>
+      </c>
+      <c r="F53" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G53" s="7" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/michael-wellendorf-hansen-b3443b6</t>
+        </is>
+      </c>
+      <c r="H53" s="7" t="inlineStr">
+        <is>
+          <t>Central DK</t>
         </is>
       </c>
     </row>
@@ -10662,32 +10873,37 @@
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>CEO/MD</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>Henning</t>
+          <t>Danny Oddershede</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>Pe***n</t>
+          <t>Engineering Manager</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t>Managing Director / CEO</t>
-        </is>
-      </c>
-      <c r="F54" s="5" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>danny.oddershede@baader.com</t>
+        </is>
+      </c>
+      <c r="F54" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G54" s="5" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/danny-o-206909130</t>
+        </is>
+      </c>
+      <c r="H54" s="5" t="inlineStr">
+        <is>
+          <t>Horsens, DK</t>
         </is>
       </c>
     </row>
@@ -10699,32 +10915,37 @@
       </c>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>R&amp;D</t>
+          <t>Production</t>
         </is>
       </c>
       <c r="C55" s="7" t="inlineStr">
         <is>
-          <t>Michael</t>
+          <t>Niels Thomassen</t>
         </is>
       </c>
       <c r="D55" s="7" t="inlineStr">
         <is>
-          <t>Ha***n</t>
+          <t>Production Manager</t>
         </is>
       </c>
       <c r="E55" s="7" t="inlineStr">
         <is>
-          <t>Head of R&amp;D</t>
-        </is>
-      </c>
-      <c r="F55" s="7" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>niels.thomassen@baader.com</t>
+        </is>
+      </c>
+      <c r="F55" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G55" s="7" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/niels-thomassen-65101464</t>
+        </is>
+      </c>
+      <c r="H55" s="7" t="inlineStr">
+        <is>
+          <t>Central DK</t>
         </is>
       </c>
     </row>
@@ -10736,76 +10957,86 @@
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>Technical Director</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>Danny</t>
+          <t>Michael Bang</t>
         </is>
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>Od***e</t>
+          <t>Technical Director</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t>Engineering Manager</t>
-        </is>
-      </c>
-      <c r="F56" s="5" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>michael.bang@baader.com</t>
+        </is>
+      </c>
+      <c r="F56" s="14" t="inlineStr">
+        <is>
+          <t>extrapolated</t>
         </is>
       </c>
       <c r="G56" s="5" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/michael-bang-8901a4b</t>
+        </is>
+      </c>
+      <c r="H56" s="5" t="inlineStr">
+        <is>
+          <t>Central DK</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
         <is>
-          <t>BAADER Food Systems Denmark A/S (ex-LINCO)</t>
+          <t>Jorgensen Engineering A/S</t>
         </is>
       </c>
       <c r="B57" s="7" t="inlineStr">
         <is>
-          <t>Production</t>
+          <t>CEO/MD</t>
         </is>
       </c>
       <c r="C57" s="7" t="inlineStr">
         <is>
-          <t>Niels</t>
+          <t>Mike Gornitzka</t>
         </is>
       </c>
       <c r="D57" s="7" t="inlineStr">
         <is>
-          <t>Th***n</t>
+          <t>Chief Executive Officer</t>
         </is>
       </c>
       <c r="E57" s="7" t="inlineStr">
         <is>
-          <t>Production Manager</t>
-        </is>
-      </c>
-      <c r="F57" s="7" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>mg@jorgensen.dk</t>
+        </is>
+      </c>
+      <c r="F57" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G57" s="7" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/mike-l-gornitzka-24a7a957</t>
+        </is>
+      </c>
+      <c r="H57" s="7" t="inlineStr">
+        <is>
+          <t>Odense, DK</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="5" t="inlineStr">
         <is>
-          <t>BAADER Food Systems Denmark A/S (ex-LINCO)</t>
+          <t>Jorgensen Engineering A/S</t>
         </is>
       </c>
       <c r="B58" s="5" t="inlineStr">
@@ -10815,27 +11046,32 @@
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>Michael</t>
+          <t>Thomas Lassen</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>Ba***g</t>
+          <t>Chief Technology Officer</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
         <is>
-          <t>Technical Director</t>
-        </is>
-      </c>
-      <c r="F58" s="5" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>tla@jorgensen.dk</t>
+        </is>
+      </c>
+      <c r="F58" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G58" s="5" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/thomas-lassen-a3b36816</t>
+        </is>
+      </c>
+      <c r="H58" s="5" t="inlineStr">
+        <is>
+          <t>Odense, DK</t>
         </is>
       </c>
     </row>
@@ -10847,32 +11083,37 @@
       </c>
       <c r="B59" s="7" t="inlineStr">
         <is>
-          <t>CEO/MD</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="C59" s="7" t="inlineStr">
         <is>
-          <t>Mike</t>
+          <t>Jeppe Johnsen</t>
         </is>
       </c>
       <c r="D59" s="7" t="inlineStr">
         <is>
-          <t>Go***a</t>
+          <t>Engineering Manager</t>
         </is>
       </c>
       <c r="E59" s="7" t="inlineStr">
         <is>
-          <t>Chief Executive Officer</t>
-        </is>
-      </c>
-      <c r="F59" s="7" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>jdj@jorgensen.dk</t>
+        </is>
+      </c>
+      <c r="F59" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G59" s="7" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/jeppe-johnsen-48665718</t>
+        </is>
+      </c>
+      <c r="H59" s="7" t="inlineStr">
+        <is>
+          <t>S. Denmark</t>
         </is>
       </c>
     </row>
@@ -10884,39 +11125,40 @@
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>Technical Director</t>
+          <t>Production</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Johnni Hansen</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>La***n</t>
-        </is>
-      </c>
-      <c r="E60" s="5" t="inlineStr">
-        <is>
-          <t>Chief Technology Officer</t>
-        </is>
-      </c>
-      <c r="F60" s="5" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>Production Manager</t>
+        </is>
+      </c>
+      <c r="E60" s="5" t="inlineStr"/>
+      <c r="F60" s="13" t="inlineStr">
+        <is>
+          <t>unavailable</t>
         </is>
       </c>
       <c r="G60" s="5" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/johnni-lysemose-hansen-148246171</t>
+        </is>
+      </c>
+      <c r="H60" s="5" t="inlineStr">
+        <is>
+          <t>S. Denmark</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
         <is>
-          <t>Jorgensen Engineering A/S</t>
+          <t>Haarslev Industries A/S</t>
         </is>
       </c>
       <c r="B61" s="7" t="inlineStr">
@@ -10926,64 +11168,70 @@
       </c>
       <c r="C61" s="7" t="inlineStr">
         <is>
-          <t>Jeppe</t>
+          <t>Kaare Vegeberg</t>
         </is>
       </c>
       <c r="D61" s="7" t="inlineStr">
         <is>
-          <t>Jo***n</t>
-        </is>
-      </c>
-      <c r="E61" s="7" t="inlineStr">
-        <is>
-          <t>Engineering Manager</t>
-        </is>
-      </c>
-      <c r="F61" s="7" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>Engineering Centre Manager</t>
+        </is>
+      </c>
+      <c r="E61" s="7" t="inlineStr"/>
+      <c r="F61" s="13" t="inlineStr">
+        <is>
+          <t>unavailable</t>
         </is>
       </c>
       <c r="G61" s="7" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/kaare-bek-vegeberg-4a3b5742</t>
+        </is>
+      </c>
+      <c r="H61" s="7" t="inlineStr">
+        <is>
+          <t>Aarup, DK</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
         <is>
-          <t>Jorgensen Engineering A/S</t>
+          <t>Haarslev Industries A/S</t>
         </is>
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>Production</t>
+          <t>Engineering (Automation)</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>Johnni</t>
+          <t>Henrik Jensen</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>Ha***n</t>
+          <t>Engineering Centre Manager, Automation &amp; Control</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t>Production Manager</t>
-        </is>
-      </c>
-      <c r="F62" s="5" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>henrik.jensen@haarslev.com</t>
+        </is>
+      </c>
+      <c r="F62" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G62" s="5" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/henrik-granly-jensen-140302a</t>
+        </is>
+      </c>
+      <c r="H62" s="5" t="inlineStr">
+        <is>
+          <t>S. Denmark</t>
         </is>
       </c>
     </row>
@@ -10995,113 +11243,120 @@
       </c>
       <c r="B63" s="7" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>Sales Engineering</t>
         </is>
       </c>
       <c r="C63" s="7" t="inlineStr">
         <is>
-          <t>Kaare</t>
+          <t>Hamed Shokoohi</t>
         </is>
       </c>
       <c r="D63" s="7" t="inlineStr">
         <is>
-          <t>Ve***g</t>
-        </is>
-      </c>
-      <c r="E63" s="7" t="inlineStr">
-        <is>
-          <t>Engineering Centre Manager</t>
-        </is>
-      </c>
-      <c r="F63" s="7" t="inlineStr">
+          <t>Sales Engineering Manager</t>
+        </is>
+      </c>
+      <c r="E63" s="7" t="inlineStr"/>
+      <c r="F63" s="13" t="inlineStr">
+        <is>
+          <t>unavailable</t>
+        </is>
+      </c>
+      <c r="G63" s="7" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/hamed-shokoohi-69b29a78</t>
+        </is>
+      </c>
+      <c r="H63" s="7" t="inlineStr">
         <is>
           <t>Denmark</t>
-        </is>
-      </c>
-      <c r="G63" s="7" t="inlineStr">
-        <is>
-          <t>(enrich to reveal)</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
         <is>
-          <t>Haarslev Industries A/S</t>
+          <t>Daniatech ApS / SD Mixing (SiccaDania)</t>
         </is>
       </c>
       <c r="B64" s="5" t="inlineStr">
         <is>
-          <t>Engineering (Automation)</t>
+          <t>CEO/MD</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>Henrik</t>
+          <t>Jens Andersen</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>Je***n</t>
+          <t>Managing Director</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
         <is>
-          <t>Engineering Centre Manager - Automation &amp; Control</t>
-        </is>
-      </c>
-      <c r="F64" s="5" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>jens.andersen@daniatech.com</t>
+        </is>
+      </c>
+      <c r="F64" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G64" s="5" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/jensnygaardandersen</t>
+        </is>
+      </c>
+      <c r="H64" s="5" t="inlineStr">
+        <is>
+          <t>Aarhus, DK</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
         <is>
-          <t>Haarslev Industries A/S</t>
+          <t>Daniatech ApS / SD Mixing (SiccaDania)</t>
         </is>
       </c>
       <c r="B65" s="7" t="inlineStr">
         <is>
-          <t>Sales Engineering</t>
+          <t>R&amp;D/Technical</t>
         </is>
       </c>
       <c r="C65" s="7" t="inlineStr">
         <is>
-          <t>Hamed</t>
+          <t>Gorm Kjaerulff</t>
         </is>
       </c>
       <c r="D65" s="7" t="inlineStr">
         <is>
-          <t>Sh***i</t>
-        </is>
-      </c>
-      <c r="E65" s="7" t="inlineStr">
-        <is>
-          <t>Sales Engineering Manager</t>
-        </is>
-      </c>
-      <c r="F65" s="7" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>Technology Owner, UHT &amp; Thermal Processing</t>
+        </is>
+      </c>
+      <c r="E65" s="7" t="inlineStr"/>
+      <c r="F65" s="13" t="inlineStr">
+        <is>
+          <t>unavailable</t>
         </is>
       </c>
       <c r="G65" s="7" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/gorm-bro-kjaerulff-0bab221b</t>
+        </is>
+      </c>
+      <c r="H65" s="7" t="inlineStr">
+        <is>
+          <t>Central DK</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="5" t="inlineStr">
         <is>
-          <t>Daniatech ApS / SD Mixing (SiccaDania)</t>
+          <t>SANOVO Technology A/S</t>
         </is>
       </c>
       <c r="B66" s="5" t="inlineStr">
@@ -11111,64 +11366,74 @@
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>Jens</t>
+          <t>Michael Midskov</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>An***n</t>
+          <t>CEO (Group)</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t>Managing Director</t>
-        </is>
-      </c>
-      <c r="F66" s="5" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>msm@sanovogroup.com</t>
+        </is>
+      </c>
+      <c r="F66" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G66" s="5" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/michael-strange-midskov-1199b621</t>
+        </is>
+      </c>
+      <c r="H66" s="5" t="inlineStr">
+        <is>
+          <t>S. Denmark</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
         <is>
-          <t>Daniatech ApS / SD Mixing (SiccaDania)</t>
+          <t>SANOVO Technology A/S</t>
         </is>
       </c>
       <c r="B67" s="7" t="inlineStr">
         <is>
-          <t>R&amp;D/Technical</t>
+          <t>R&amp;D</t>
         </is>
       </c>
       <c r="C67" s="7" t="inlineStr">
         <is>
-          <t>Gorm</t>
+          <t>Martin Sorensen</t>
         </is>
       </c>
       <c r="D67" s="7" t="inlineStr">
         <is>
-          <t>Kj***f</t>
+          <t>R&amp;D Manager</t>
         </is>
       </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
-          <t>Technology Owner, UHT &amp; Thermal Processing</t>
-        </is>
-      </c>
-      <c r="F67" s="7" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>mas@sanovogroup.com</t>
+        </is>
+      </c>
+      <c r="F67" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G67" s="7" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/martin-sørensen-39ba96139</t>
+        </is>
+      </c>
+      <c r="H67" s="7" t="inlineStr">
+        <is>
+          <t>Odense, DK</t>
         </is>
       </c>
     </row>
@@ -11180,106 +11445,117 @@
       </c>
       <c r="B68" s="5" t="inlineStr">
         <is>
-          <t>CEO/MD</t>
+          <t>Engineering (Electrical)</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>Michael</t>
+          <t>Henrik Moller</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>Mi***v</t>
-        </is>
-      </c>
-      <c r="E68" s="5" t="inlineStr">
-        <is>
-          <t>CEO</t>
-        </is>
-      </c>
-      <c r="F68" s="5" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>Product Owner, Electrical</t>
+        </is>
+      </c>
+      <c r="E68" s="5" t="inlineStr"/>
+      <c r="F68" s="13" t="inlineStr">
+        <is>
+          <t>unavailable</t>
         </is>
       </c>
       <c r="G68" s="5" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/henrik-møller-93b09b84</t>
+        </is>
+      </c>
+      <c r="H68" s="5" t="inlineStr">
+        <is>
+          <t>Svendborg, DK</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="7" t="inlineStr">
         <is>
-          <t>SANOVO Technology A/S</t>
+          <t>Scanvaegt Systems A/S</t>
         </is>
       </c>
       <c r="B69" s="7" t="inlineStr">
         <is>
-          <t>R&amp;D</t>
+          <t>CEO/MD</t>
         </is>
       </c>
       <c r="C69" s="7" t="inlineStr">
         <is>
-          <t>Martin</t>
+          <t>Jan Elgaard</t>
         </is>
       </c>
       <c r="D69" s="7" t="inlineStr">
         <is>
-          <t>So***n</t>
+          <t>Adm. Direktor / CEO</t>
         </is>
       </c>
       <c r="E69" s="7" t="inlineStr">
         <is>
-          <t>R&amp;D Manager</t>
-        </is>
-      </c>
-      <c r="F69" s="7" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>jel@scanvaegt.dk</t>
+        </is>
+      </c>
+      <c r="F69" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G69" s="7" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/jan-elgaard-34bab22</t>
+        </is>
+      </c>
+      <c r="H69" s="7" t="inlineStr">
+        <is>
+          <t>Aarhus, DK</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="5" t="inlineStr">
         <is>
-          <t>SANOVO Technology A/S</t>
+          <t>Scanvaegt Systems A/S</t>
         </is>
       </c>
       <c r="B70" s="5" t="inlineStr">
         <is>
-          <t>Engineering (Electrical)</t>
+          <t>R&amp;D</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>Henrik</t>
+          <t>Simon Sogaard</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>Mo***r</t>
+          <t>R&amp;D Team Manager</t>
         </is>
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t>Product Owner, Electrical</t>
-        </is>
-      </c>
-      <c r="F70" s="5" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>s.sogaard@scanvaegt.com</t>
+        </is>
+      </c>
+      <c r="F70" s="14" t="inlineStr">
+        <is>
+          <t>extrapolated</t>
         </is>
       </c>
       <c r="G70" s="5" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/simon-vejlin-søgaard-4278825a</t>
+        </is>
+      </c>
+      <c r="H70" s="5" t="inlineStr">
+        <is>
+          <t>Aarhus, DK</t>
         </is>
       </c>
     </row>
@@ -11291,106 +11567,117 @@
       </c>
       <c r="B71" s="7" t="inlineStr">
         <is>
-          <t>CEO/MD</t>
+          <t>R&amp;D (Project)</t>
         </is>
       </c>
       <c r="C71" s="7" t="inlineStr">
         <is>
-          <t>Jan</t>
+          <t>Niels Hundtofte</t>
         </is>
       </c>
       <c r="D71" s="7" t="inlineStr">
         <is>
-          <t>El***d</t>
-        </is>
-      </c>
-      <c r="E71" s="7" t="inlineStr">
-        <is>
-          <t>Adm. Direktor / CEO</t>
-        </is>
-      </c>
-      <c r="F71" s="7" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>Project Manager R&amp;D</t>
+        </is>
+      </c>
+      <c r="E71" s="7" t="inlineStr"/>
+      <c r="F71" s="13" t="inlineStr">
+        <is>
+          <t>unavailable</t>
         </is>
       </c>
       <c r="G71" s="7" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/niels-hundtofte-8719056</t>
+        </is>
+      </c>
+      <c r="H71" s="7" t="inlineStr">
+        <is>
+          <t>Central DK</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="5" t="inlineStr">
         <is>
-          <t>Scanvaegt Systems A/S</t>
+          <t>Schur Technology A/S (Schur Group)</t>
         </is>
       </c>
       <c r="B72" s="5" t="inlineStr">
         <is>
-          <t>R&amp;D</t>
+          <t>CEO/MD</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>Simon</t>
+          <t>Hans Schur</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>So***d</t>
+          <t>Chief Executive Officer</t>
         </is>
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
-          <t>R&amp;D Team Manager</t>
-        </is>
-      </c>
-      <c r="F72" s="5" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>hcs@schur.com</t>
+        </is>
+      </c>
+      <c r="F72" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/hans-christian-schur-45a69a14</t>
+        </is>
+      </c>
+      <c r="H72" s="5" t="inlineStr">
+        <is>
+          <t>Central DK</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="7" t="inlineStr">
         <is>
-          <t>Scanvaegt Systems A/S</t>
+          <t>Schur Technology A/S (Schur Group)</t>
         </is>
       </c>
       <c r="B73" s="7" t="inlineStr">
         <is>
-          <t>R&amp;D (Project)</t>
+          <t>Purchasing</t>
         </is>
       </c>
       <c r="C73" s="7" t="inlineStr">
         <is>
-          <t>Niels</t>
+          <t>Kasper Andersen</t>
         </is>
       </c>
       <c r="D73" s="7" t="inlineStr">
         <is>
-          <t>Hu***e</t>
+          <t>Procurement Manager</t>
         </is>
       </c>
       <c r="E73" s="7" t="inlineStr">
         <is>
-          <t>Project Manager R&amp;D</t>
-        </is>
-      </c>
-      <c r="F73" s="7" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>kfa@schur.com</t>
+        </is>
+      </c>
+      <c r="F73" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G73" s="7" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/kasper-andersen-97574225</t>
+        </is>
+      </c>
+      <c r="H73" s="7" t="inlineStr">
+        <is>
+          <t>S. Denmark</t>
         </is>
       </c>
     </row>
@@ -11402,32 +11689,37 @@
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>CEO/MD</t>
+          <t>Supply Chain</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>Hans</t>
+          <t>Ditte Christensen</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>Sc***r</t>
+          <t>Director of Supply Chain</t>
         </is>
       </c>
       <c r="E74" s="5" t="inlineStr">
         <is>
-          <t>Chief Executive Officer</t>
-        </is>
-      </c>
-      <c r="F74" s="5" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>dch@schur.com</t>
+        </is>
+      </c>
+      <c r="F74" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/ditte-christensen-831a1174</t>
+        </is>
+      </c>
+      <c r="H74" s="5" t="inlineStr">
+        <is>
+          <t>Horsens, DK</t>
         </is>
       </c>
     </row>
@@ -11439,106 +11731,117 @@
       </c>
       <c r="B75" s="7" t="inlineStr">
         <is>
-          <t>Purchasing/Procurement</t>
+          <t>Production</t>
         </is>
       </c>
       <c r="C75" s="7" t="inlineStr">
         <is>
-          <t>Kasper</t>
+          <t>Michael Trebbien</t>
         </is>
       </c>
       <c r="D75" s="7" t="inlineStr">
         <is>
-          <t>An***n</t>
-        </is>
-      </c>
-      <c r="E75" s="7" t="inlineStr">
-        <is>
-          <t>Procurement Manager</t>
-        </is>
-      </c>
-      <c r="F75" s="7" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>Produktions Leder</t>
+        </is>
+      </c>
+      <c r="E75" s="7" t="inlineStr"/>
+      <c r="F75" s="13" t="inlineStr">
+        <is>
+          <t>unavailable</t>
         </is>
       </c>
       <c r="G75" s="7" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/michael-trebbien-37451927</t>
+        </is>
+      </c>
+      <c r="H75" s="7" t="inlineStr">
+        <is>
+          <t>Vejle, DK</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="5" t="inlineStr">
         <is>
-          <t>Schur Technology A/S (Schur Group)</t>
+          <t>Aasted ApS</t>
         </is>
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>Supply Chain</t>
+          <t>CEO/MD</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>Ditte</t>
+          <t>Piet Taestensen</t>
         </is>
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>Ch***n</t>
+          <t>CEO</t>
         </is>
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t>Director of Supply Chain</t>
-        </is>
-      </c>
-      <c r="F76" s="5" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>piet.taestensen@aasted.eu</t>
+        </is>
+      </c>
+      <c r="F76" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G76" s="5" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/piettaestensen</t>
+        </is>
+      </c>
+      <c r="H76" s="5" t="inlineStr">
+        <is>
+          <t>Zealand, DK</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="7" t="inlineStr">
         <is>
-          <t>Schur Technology A/S (Schur Group)</t>
+          <t>Aasted ApS</t>
         </is>
       </c>
       <c r="B77" s="7" t="inlineStr">
         <is>
-          <t>Production</t>
+          <t>Technical Director/CTO</t>
         </is>
       </c>
       <c r="C77" s="7" t="inlineStr">
         <is>
-          <t>Michael</t>
+          <t>Henrik Heitmann</t>
         </is>
       </c>
       <c r="D77" s="7" t="inlineStr">
         <is>
-          <t>Tr***n</t>
+          <t>Chief Technology Officer</t>
         </is>
       </c>
       <c r="E77" s="7" t="inlineStr">
         <is>
-          <t>Produktions Leder</t>
-        </is>
-      </c>
-      <c r="F77" s="7" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>henrik.heitmann@aasted.eu</t>
+        </is>
+      </c>
+      <c r="F77" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G77" s="7" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/henrikheitmann</t>
+        </is>
+      </c>
+      <c r="H77" s="7" t="inlineStr">
+        <is>
+          <t>Hoje Taastrup, DK</t>
         </is>
       </c>
     </row>
@@ -11550,32 +11853,37 @@
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>CEO/MD</t>
+          <t>Purchasing</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>Piet</t>
+          <t>Christian Aasted</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>Ta***n</t>
+          <t>Head of Purchasing Department</t>
         </is>
       </c>
       <c r="E78" s="5" t="inlineStr">
         <is>
-          <t>CEO</t>
-        </is>
-      </c>
-      <c r="F78" s="5" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>christian.aasted@aasted.eu</t>
+        </is>
+      </c>
+      <c r="F78" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G78" s="5" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/christianaasted</t>
+        </is>
+      </c>
+      <c r="H78" s="5" t="inlineStr">
+        <is>
+          <t>Copenhagen, DK</t>
         </is>
       </c>
     </row>
@@ -11587,32 +11895,33 @@
       </c>
       <c r="B79" s="7" t="inlineStr">
         <is>
-          <t>Technical Director/CTO</t>
+          <t>Production</t>
         </is>
       </c>
       <c r="C79" s="7" t="inlineStr">
         <is>
-          <t>Henrik</t>
+          <t>Paw Nedahl</t>
         </is>
       </c>
       <c r="D79" s="7" t="inlineStr">
         <is>
-          <t>He***n</t>
-        </is>
-      </c>
-      <c r="E79" s="7" t="inlineStr">
-        <is>
-          <t>Chief Technology Officer</t>
-        </is>
-      </c>
-      <c r="F79" s="7" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>Production Manager</t>
+        </is>
+      </c>
+      <c r="E79" s="7" t="inlineStr"/>
+      <c r="F79" s="13" t="inlineStr">
+        <is>
+          <t>unavailable</t>
         </is>
       </c>
       <c r="G79" s="7" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/paw-boris-nedahl-329bb413a</t>
+        </is>
+      </c>
+      <c r="H79" s="7" t="inlineStr">
+        <is>
+          <t>Copenhagen, DK</t>
         </is>
       </c>
     </row>
@@ -11624,32 +11933,37 @@
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>Purchasing</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>Christian</t>
+          <t>Niels Hansen</t>
         </is>
       </c>
       <c r="D80" s="5" t="inlineStr">
         <is>
-          <t>Aa***d</t>
+          <t>Head of Sales Engineering</t>
         </is>
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t>Head of Purchasing Department</t>
-        </is>
-      </c>
-      <c r="F80" s="5" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>niels.hansen@aasted.eu</t>
+        </is>
+      </c>
+      <c r="F80" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G80" s="5" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/niels-schmidt-hansen-04b21a85</t>
+        </is>
+      </c>
+      <c r="H80" s="5" t="inlineStr">
+        <is>
+          <t>Copenhagen, DK</t>
         </is>
       </c>
     </row>
@@ -11661,217 +11975,243 @@
       </c>
       <c r="B81" s="7" t="inlineStr">
         <is>
-          <t>Production</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="C81" s="7" t="inlineStr">
         <is>
-          <t>Paw</t>
+          <t>Allan Aasted</t>
         </is>
       </c>
       <c r="D81" s="7" t="inlineStr">
         <is>
-          <t>Ne***l</t>
+          <t>Vice Chairman, Owner</t>
         </is>
       </c>
       <c r="E81" s="7" t="inlineStr">
         <is>
-          <t>Production Manager</t>
-        </is>
-      </c>
-      <c r="F81" s="7" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>allan.aasted@aasted.eu</t>
+        </is>
+      </c>
+      <c r="F81" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G81" s="7" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/allanaasted</t>
+        </is>
+      </c>
+      <c r="H81" s="7" t="inlineStr">
+        <is>
+          <t>Farum, DK</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="5" t="inlineStr">
         <is>
-          <t>Aasted ApS</t>
+          <t>Varimixer A/S (Wodschow &amp; Co.)</t>
         </is>
       </c>
       <c r="B82" s="5" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>CEO/MD</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>Niels</t>
+          <t>Paw Soe</t>
         </is>
       </c>
       <c r="D82" s="5" t="inlineStr">
         <is>
-          <t>Ha***n</t>
+          <t>CEO</t>
         </is>
       </c>
       <c r="E82" s="5" t="inlineStr">
         <is>
-          <t>Head of Sales Engineering</t>
-        </is>
-      </c>
-      <c r="F82" s="5" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>paw.soe@varimixer.com</t>
+        </is>
+      </c>
+      <c r="F82" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G82" s="5" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/paw-søe-60a0b4408</t>
+        </is>
+      </c>
+      <c r="H82" s="5" t="inlineStr">
+        <is>
+          <t>Copenhagen, DK</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="7" t="inlineStr">
         <is>
-          <t>Aasted ApS</t>
+          <t>Varimixer A/S (Wodschow &amp; Co.)</t>
         </is>
       </c>
       <c r="B83" s="7" t="inlineStr">
         <is>
-          <t>Owner</t>
+          <t>Production</t>
         </is>
       </c>
       <c r="C83" s="7" t="inlineStr">
         <is>
-          <t>Allan</t>
+          <t>Jesper Olsen</t>
         </is>
       </c>
       <c r="D83" s="7" t="inlineStr">
         <is>
-          <t>Aa***d</t>
+          <t>Production Manager</t>
         </is>
       </c>
       <c r="E83" s="7" t="inlineStr">
         <is>
-          <t>Vice Chairman, Owner</t>
-        </is>
-      </c>
-      <c r="F83" s="7" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>jesper.olsen@varimixer.com</t>
+        </is>
+      </c>
+      <c r="F83" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G83" s="7" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/jesper-olsen-610b74260</t>
+        </is>
+      </c>
+      <c r="H83" s="7" t="inlineStr">
+        <is>
+          <t>Copenhagen, DK</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="5" t="inlineStr">
         <is>
-          <t>Varimixer A/S (Wodschow &amp; Co.)</t>
+          <t>Chocoma ApS</t>
         </is>
       </c>
       <c r="B84" s="5" t="inlineStr">
         <is>
-          <t>CEO/MD</t>
+          <t>CEO/MD (Owner)</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
         <is>
-          <t>Paw</t>
+          <t>Christian Nilsson</t>
         </is>
       </c>
       <c r="D84" s="5" t="inlineStr">
         <is>
-          <t>Soe</t>
+          <t>Owner</t>
         </is>
       </c>
       <c r="E84" s="5" t="inlineStr">
         <is>
-          <t>CEO</t>
-        </is>
-      </c>
-      <c r="F84" s="5" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>cn@chocoma.com</t>
+        </is>
+      </c>
+      <c r="F84" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G84" s="5" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/christian-nilsson-60b615135</t>
+        </is>
+      </c>
+      <c r="H84" s="5" t="inlineStr">
+        <is>
+          <t>Capital Region, DK</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="7" t="inlineStr">
         <is>
-          <t>Varimixer A/S (Wodschow &amp; Co.)</t>
+          <t>Sealing System 2024 A/S</t>
         </is>
       </c>
       <c r="B85" s="7" t="inlineStr">
         <is>
-          <t>Production</t>
+          <t>CEO/MD</t>
         </is>
       </c>
       <c r="C85" s="7" t="inlineStr">
         <is>
-          <t>Jesper</t>
+          <t>Ole Jensen</t>
         </is>
       </c>
       <c r="D85" s="7" t="inlineStr">
         <is>
-          <t>Ol***n</t>
-        </is>
-      </c>
-      <c r="E85" s="7" t="inlineStr">
-        <is>
-          <t>Production Manager</t>
-        </is>
-      </c>
-      <c r="F85" s="7" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="E85" s="7" t="inlineStr"/>
+      <c r="F85" s="13" t="inlineStr">
+        <is>
+          <t>unavailable</t>
         </is>
       </c>
       <c r="G85" s="7" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/ole-jensen-</t>
+        </is>
+      </c>
+      <c r="H85" s="7" t="inlineStr">
+        <is>
+          <t>Copenhagen, DK</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="5" t="inlineStr">
         <is>
-          <t>Chocoma ApS</t>
+          <t>Sealing System 2024 A/S</t>
         </is>
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>CEO/MD (Owner)</t>
+          <t>Purchasing</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
         <is>
-          <t>Christian</t>
+          <t>Dion Lauridsen</t>
         </is>
       </c>
       <c r="D86" s="5" t="inlineStr">
         <is>
-          <t>Ni***n</t>
+          <t>Procurement Manager</t>
         </is>
       </c>
       <c r="E86" s="5" t="inlineStr">
         <is>
-          <t>Owner</t>
-        </is>
-      </c>
-      <c r="F86" s="5" t="inlineStr">
+          <t>dla@sealing-system.dk</t>
+        </is>
+      </c>
+      <c r="F86" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="G86" s="5" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/dion-lauridsen-bb4803b</t>
+        </is>
+      </c>
+      <c r="H86" s="5" t="inlineStr">
         <is>
           <t>Denmark</t>
-        </is>
-      </c>
-      <c r="G86" s="5" t="inlineStr">
-        <is>
-          <t>(enrich to reveal)</t>
         </is>
       </c>
     </row>
@@ -11883,32 +12223,33 @@
       </c>
       <c r="B87" s="7" t="inlineStr">
         <is>
-          <t>CEO/MD</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="C87" s="7" t="inlineStr">
         <is>
-          <t>Ole</t>
+          <t>Tonny Raunsbaek</t>
         </is>
       </c>
       <c r="D87" s="7" t="inlineStr">
         <is>
-          <t>Je***n</t>
-        </is>
-      </c>
-      <c r="E87" s="7" t="inlineStr">
-        <is>
-          <t>CEO</t>
-        </is>
-      </c>
-      <c r="F87" s="7" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>Engineering Manager</t>
+        </is>
+      </c>
+      <c r="E87" s="7" t="inlineStr"/>
+      <c r="F87" s="13" t="inlineStr">
+        <is>
+          <t>unavailable</t>
         </is>
       </c>
       <c r="G87" s="7" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/tonny-raunsbæk-b87ba3123</t>
+        </is>
+      </c>
+      <c r="H87" s="7" t="inlineStr">
+        <is>
+          <t>S. Denmark</t>
         </is>
       </c>
     </row>
@@ -11920,32 +12261,33 @@
       </c>
       <c r="B88" s="5" t="inlineStr">
         <is>
-          <t>Purchasing/Procurement</t>
+          <t>Technical Director</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
         <is>
-          <t>Dion</t>
+          <t>Tue Pedersen</t>
         </is>
       </c>
       <c r="D88" s="5" t="inlineStr">
         <is>
-          <t>La***n</t>
-        </is>
-      </c>
-      <c r="E88" s="5" t="inlineStr">
-        <is>
-          <t>Procurement Manager</t>
-        </is>
-      </c>
-      <c r="F88" s="5" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>Technical Director</t>
+        </is>
+      </c>
+      <c r="E88" s="5" t="inlineStr"/>
+      <c r="F88" s="13" t="inlineStr">
+        <is>
+          <t>unavailable</t>
         </is>
       </c>
       <c r="G88" s="5" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/tue-pedersen-47549182</t>
+        </is>
+      </c>
+      <c r="H88" s="5" t="inlineStr">
+        <is>
+          <t>Give, DK</t>
         </is>
       </c>
     </row>
@@ -11957,143 +12299,163 @@
       </c>
       <c r="B89" s="7" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>Production</t>
         </is>
       </c>
       <c r="C89" s="7" t="inlineStr">
         <is>
-          <t>Tonny</t>
+          <t>Rasmus Danielsen</t>
         </is>
       </c>
       <c r="D89" s="7" t="inlineStr">
         <is>
-          <t>Ra***k</t>
+          <t>Manager of Electrical Engineering &amp; Manufacturing</t>
         </is>
       </c>
       <c r="E89" s="7" t="inlineStr">
         <is>
-          <t>Engineering Manager</t>
-        </is>
-      </c>
-      <c r="F89" s="7" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>rda@sealing-system.dk</t>
+        </is>
+      </c>
+      <c r="F89" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G89" s="7" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/rasmus-danielsen</t>
+        </is>
+      </c>
+      <c r="H89" s="7" t="inlineStr">
+        <is>
+          <t>S. Denmark</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="5" t="inlineStr">
         <is>
-          <t>Sealing System 2024 A/S</t>
+          <t>Dansk Maskin Teknik A/S (DMT)</t>
         </is>
       </c>
       <c r="B90" s="5" t="inlineStr">
         <is>
-          <t>Technical Director</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>Tue</t>
+          <t>Andreas Landsfeldt-Erichsen</t>
         </is>
       </c>
       <c r="D90" s="5" t="inlineStr">
         <is>
-          <t>Pe***n</t>
+          <t>Head of Mechanical Engineering</t>
         </is>
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t>Technical Director</t>
-        </is>
-      </c>
-      <c r="F90" s="5" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>al@dmt-as.dk</t>
+        </is>
+      </c>
+      <c r="F90" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G90" s="5" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/andreas-landsfeldt-erichsen-b6707b104</t>
+        </is>
+      </c>
+      <c r="H90" s="5" t="inlineStr">
+        <is>
+          <t>Ryomgård, DK</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="7" t="inlineStr">
         <is>
-          <t>Sealing System 2024 A/S</t>
+          <t>Micro Matic A/S</t>
         </is>
       </c>
       <c r="B91" s="7" t="inlineStr">
         <is>
-          <t>Production</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="C91" s="7" t="inlineStr">
         <is>
-          <t>Rasmus</t>
+          <t>Thomas Mackeprang</t>
         </is>
       </c>
       <c r="D91" s="7" t="inlineStr">
         <is>
-          <t>Da***n</t>
+          <t>Head of Engineering</t>
         </is>
       </c>
       <c r="E91" s="7" t="inlineStr">
         <is>
-          <t>Manager of Electrical Engineering &amp; Manufacturing</t>
-        </is>
-      </c>
-      <c r="F91" s="7" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>tfhm@micro-matic.dk</t>
+        </is>
+      </c>
+      <c r="F91" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G91" s="7" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/thomas-mackeprang-9931815</t>
+        </is>
+      </c>
+      <c r="H91" s="7" t="inlineStr">
+        <is>
+          <t>Odense, DK</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="5" t="inlineStr">
         <is>
-          <t>Dansk Maskin Teknik A/S (DMT)</t>
+          <t>Micro Matic A/S</t>
         </is>
       </c>
       <c r="B92" s="5" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>Purchasing</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>Andreas</t>
+          <t>Danny Lindemose</t>
         </is>
       </c>
       <c r="D92" s="5" t="inlineStr">
         <is>
-          <t>La***n</t>
+          <t>Project Manager - Group Procurement</t>
         </is>
       </c>
       <c r="E92" s="5" t="inlineStr">
         <is>
-          <t>Head of Mechanical Engineering</t>
-        </is>
-      </c>
-      <c r="F92" s="5" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>dalin@micro-matic.dk</t>
+        </is>
+      </c>
+      <c r="F92" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G92" s="5" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/danny-lindemose-5961b333</t>
+        </is>
+      </c>
+      <c r="H92" s="5" t="inlineStr">
+        <is>
+          <t>Odense, DK</t>
         </is>
       </c>
     </row>
@@ -12105,208 +12467,138 @@
       </c>
       <c r="B93" s="7" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>Production</t>
         </is>
       </c>
       <c r="C93" s="7" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Kristian Andersen</t>
         </is>
       </c>
       <c r="D93" s="7" t="inlineStr">
         <is>
-          <t>Ma***g</t>
-        </is>
-      </c>
-      <c r="E93" s="7" t="inlineStr">
-        <is>
-          <t>Head of Engineering</t>
-        </is>
-      </c>
-      <c r="F93" s="7" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>Production Manager</t>
+        </is>
+      </c>
+      <c r="E93" s="7" t="inlineStr"/>
+      <c r="F93" s="13" t="inlineStr">
+        <is>
+          <t>unavailable</t>
         </is>
       </c>
       <c r="G93" s="7" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/kristian-andersen-b809a0b</t>
+        </is>
+      </c>
+      <c r="H93" s="7" t="inlineStr">
+        <is>
+          <t>S. Denmark</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="5" t="inlineStr">
         <is>
-          <t>Micro Matic A/S</t>
+          <t>Flexmatic (now SteelXperts ApS)</t>
         </is>
       </c>
       <c r="B94" s="5" t="inlineStr">
         <is>
-          <t>Purchasing/Procurement</t>
+          <t>CEO/MD</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
         <is>
-          <t>Danny</t>
+          <t>Bjarne Sorensen</t>
         </is>
       </c>
       <c r="D94" s="5" t="inlineStr">
         <is>
-          <t>Li***e</t>
+          <t>Adm. Direktor og Medejer</t>
         </is>
       </c>
       <c r="E94" s="5" t="inlineStr">
         <is>
-          <t>Project Manager - Group Procurement</t>
-        </is>
-      </c>
-      <c r="F94" s="5" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>bs@stxp.dk</t>
+        </is>
+      </c>
+      <c r="F94" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G94" s="5" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/bjarne-sørensen-a21b7411</t>
+        </is>
+      </c>
+      <c r="H94" s="5" t="inlineStr">
+        <is>
+          <t>Holstebro, DK</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="7" t="inlineStr">
         <is>
-          <t>Micro Matic A/S</t>
+          <t>Dalum Beverage Equipment ApS</t>
         </is>
       </c>
       <c r="B95" s="7" t="inlineStr">
         <is>
-          <t>Production</t>
+          <t>CEO/MD</t>
         </is>
       </c>
       <c r="C95" s="7" t="inlineStr">
         <is>
-          <t>Kristian</t>
+          <t>Kim Dalum</t>
         </is>
       </c>
       <c r="D95" s="7" t="inlineStr">
         <is>
-          <t>An***n</t>
+          <t>CEO</t>
         </is>
       </c>
       <c r="E95" s="7" t="inlineStr">
         <is>
-          <t>Production Manager</t>
-        </is>
-      </c>
-      <c r="F95" s="7" t="inlineStr">
-        <is>
-          <t>Denmark</t>
+          <t>kim@dalumequipment.com</t>
+        </is>
+      </c>
+      <c r="F95" s="12" t="inlineStr">
+        <is>
+          <t>verified</t>
         </is>
       </c>
       <c r="G95" s="7" t="inlineStr">
         <is>
-          <t>(enrich to reveal)</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" s="5" t="inlineStr">
-        <is>
-          <t>Flexmatic (now SteelXperts ApS)</t>
-        </is>
-      </c>
-      <c r="B96" s="5" t="inlineStr">
-        <is>
-          <t>CEO/MD</t>
-        </is>
-      </c>
-      <c r="C96" s="5" t="inlineStr">
-        <is>
-          <t>Bjarne</t>
-        </is>
-      </c>
-      <c r="D96" s="5" t="inlineStr">
-        <is>
-          <t>So***n</t>
-        </is>
-      </c>
-      <c r="E96" s="5" t="inlineStr">
-        <is>
-          <t>Adm. Direktor og Medejer</t>
-        </is>
-      </c>
-      <c r="F96" s="5" t="inlineStr">
-        <is>
-          <t>Denmark</t>
-        </is>
-      </c>
-      <c r="G96" s="5" t="inlineStr">
-        <is>
-          <t>(enrich to reveal)</t>
+          <t>linkedin.com/in/kimchrdalum</t>
+        </is>
+      </c>
+      <c r="H95" s="7" t="inlineStr">
+        <is>
+          <t>Odense, DK</t>
         </is>
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="7" t="inlineStr">
-        <is>
-          <t>Dalum Beverage Equipment ApS</t>
-        </is>
-      </c>
-      <c r="B97" s="7" t="inlineStr">
-        <is>
-          <t>CEO/MD</t>
-        </is>
-      </c>
-      <c r="C97" s="7" t="inlineStr">
-        <is>
-          <t>Kim</t>
-        </is>
-      </c>
-      <c r="D97" s="7" t="inlineStr">
-        <is>
-          <t>Da***m</t>
-        </is>
-      </c>
-      <c r="E97" s="7" t="inlineStr">
-        <is>
-          <t>CEO</t>
-        </is>
-      </c>
-      <c r="F97" s="7" t="inlineStr">
-        <is>
-          <t>Denmark</t>
-        </is>
-      </c>
-      <c r="G97" s="7" t="inlineStr">
-        <is>
-          <t>(enrich to reveal)</t>
+      <c r="A97" s="15" t="inlineStr">
+        <is>
+          <t>94 decision-makers enriched via Apollo People Match. 62 verified business emails; 0 rows still enriching (Group B).</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="16" t="inlineStr">
+        <is>
+          <t>Email status: verified = confirmed deliverable; extrapolated = pattern-inferred (~medium confidence); unavailable = no email in Apollo (LinkedIn still provided).</t>
         </is>
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="12" t="inlineStr">
-        <is>
-          <t>96 decision-makers across 36 of 49 companies, pulled via Apollo People Search (FREE, no credits).</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" s="13" t="inlineStr">
-        <is>
-          <t>Last names are MASKED by Apollo (e.g. Ra***n). Full name + business email + LinkedIn URL require an</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" s="13" t="inlineStr">
-        <is>
-          <t>enrichment pass (~1 lead credit per person). 13 companies returned no Apollo records: Kroma, BoPil, Trepko,</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" s="13" t="inlineStr">
-        <is>
-          <t>Landia, CTI Process, Attec (merged into Frontmatec), Butina, DanfoTech, Skals, Bila, Haas-Meincke, Bruel, FH Scandinox.</t>
+      <c r="A99" s="16" t="inlineStr">
+        <is>
+          <t>13 companies had no Apollo records: Kroma, BoPil, Trepko, Landia, CTI Process, Attec (merged-&gt;Frontmatec), Butina, DanfoTech, Skals, Bila, Haas-Meincke, Bruel, FH Scandinox.</t>
         </is>
       </c>
     </row>
@@ -12507,7 +12799,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="A10" s="16" t="inlineStr">
         <is>
           <t>All supplier assignments in this workbook are INFERRED (no public BOM). Verify per account before outreach.</t>
         </is>

</xml_diff>